<commit_message>
trabajando en la interfaz con el usuario
</commit_message>
<xml_diff>
--- a/TRABAJOS-PYTHON/COTIZA_ALU_TEM/lista_materiales.xlsx
+++ b/TRABAJOS-PYTHON/COTIZA_ALU_TEM/lista_materiales.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PcAsusZenbookRafita\Desktop\REPO_RAFAEL_ANTEQUERA\TRABAJOS-PYTHON\COTIZA_ALU_TEM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A46660F-1F28-4383-835C-59A389EA1EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5873B4A0-1ADF-491F-8186-A083E82DF842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1B3D5D76-0D2B-4247-8E51-F5AC57810600}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1B3D5D76-0D2B-4247-8E51-F5AC57810600}"/>
   </bookViews>
   <sheets>
     <sheet name="Costo M.P.yMat." sheetId="1" r:id="rId1"/>
     <sheet name="Costo M.P.yMat. (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Costo M.P.yMat.'!$A$2:$F$94</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Costo M.P.yMat. (2)'!$A$2:$R$261</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Costo M.P.yMat. (2)'!$2:$5</definedName>
   </definedNames>
@@ -5594,6 +5595,18 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5605,18 +5618,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6276,6 +6277,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22093356-79CE-4C8B-B9F6-F910C3837076}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:O203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -6351,10 +6355,10 @@
       <c r="D3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="86" t="s">
+      <c r="E3" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="86"/>
+      <c r="F3" s="90"/>
       <c r="G3" s="48" t="s">
         <v>496</v>
       </c>
@@ -14872,8 +14876,8 @@
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="0.21" bottom="0.34" header="0" footer="0"/>
-  <pageSetup scale="60" orientation="portrait" horizontalDpi="180" verticalDpi="144"/>
-  <drawing r:id="rId1"/>
+  <pageSetup scale="82" fitToHeight="0" orientation="portrait" horizontalDpi="180" verticalDpi="144" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -15020,7 +15024,7 @@
       <c r="M3" s="47" t="s">
         <v>1530</v>
       </c>
-      <c r="N3" s="89"/>
+      <c r="N3" s="93"/>
       <c r="O3" s="47" t="s">
         <v>1</v>
       </c>
@@ -15033,10 +15037,10 @@
       <c r="R3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="S3" s="86" t="s">
+      <c r="S3" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="T3" s="86"/>
+      <c r="T3" s="90"/>
       <c r="U3" s="48" t="s">
         <v>496</v>
       </c>
@@ -15114,7 +15118,7 @@
       <c r="M4" s="49" t="s">
         <v>1282</v>
       </c>
-      <c r="N4" s="89"/>
+      <c r="N4" s="93"/>
       <c r="O4" s="49"/>
       <c r="P4" s="49" t="s">
         <v>320</v>
@@ -15164,7 +15168,7 @@
       <c r="K5" s="51"/>
       <c r="L5" s="51"/>
       <c r="M5" s="51"/>
-      <c r="N5" s="89"/>
+      <c r="N5" s="93"/>
       <c r="O5" s="51"/>
       <c r="P5" s="51"/>
       <c r="Q5" s="51"/>
@@ -15251,7 +15255,7 @@
         <f t="shared" ref="M6:M37" si="12">CONCATENATE("mp_ac[",N6,"][17]")</f>
         <v>mp_ac[0][17]</v>
       </c>
-      <c r="N6" s="90">
+      <c r="N6" s="86">
         <v>0</v>
       </c>
       <c r="O6" s="25" t="s">
@@ -15372,7 +15376,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[1][17]</v>
       </c>
-      <c r="N7" s="90">
+      <c r="N7" s="86">
         <v>1</v>
       </c>
       <c r="O7" s="11" t="s">
@@ -15498,7 +15502,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[2][17]</v>
       </c>
-      <c r="N8" s="90">
+      <c r="N8" s="86">
         <v>2</v>
       </c>
       <c r="O8" s="11" t="s">
@@ -15624,7 +15628,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[3][17]</v>
       </c>
-      <c r="N9" s="90">
+      <c r="N9" s="86">
         <v>3</v>
       </c>
       <c r="O9" s="11" t="s">
@@ -15750,7 +15754,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[4][17]</v>
       </c>
-      <c r="N10" s="90">
+      <c r="N10" s="86">
         <v>4</v>
       </c>
       <c r="O10" s="11" t="s">
@@ -15876,7 +15880,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[5][17]</v>
       </c>
-      <c r="N11" s="90">
+      <c r="N11" s="86">
         <v>5</v>
       </c>
       <c r="O11" s="11" t="s">
@@ -16002,7 +16006,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[6][17]</v>
       </c>
-      <c r="N12" s="90">
+      <c r="N12" s="86">
         <v>6</v>
       </c>
       <c r="O12" s="11" t="s">
@@ -16128,7 +16132,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[7][17]</v>
       </c>
-      <c r="N13" s="90">
+      <c r="N13" s="86">
         <v>7</v>
       </c>
       <c r="O13" s="11" t="s">
@@ -16254,7 +16258,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[8][17]</v>
       </c>
-      <c r="N14" s="90">
+      <c r="N14" s="86">
         <v>8</v>
       </c>
       <c r="O14" s="11" t="s">
@@ -16380,7 +16384,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[9][17]</v>
       </c>
-      <c r="N15" s="90">
+      <c r="N15" s="86">
         <v>9</v>
       </c>
       <c r="O15" s="11" t="s">
@@ -16506,7 +16510,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[10][17]</v>
       </c>
-      <c r="N16" s="90">
+      <c r="N16" s="86">
         <v>10</v>
       </c>
       <c r="O16" s="11" t="s">
@@ -16632,7 +16636,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[11][17]</v>
       </c>
-      <c r="N17" s="90">
+      <c r="N17" s="86">
         <v>11</v>
       </c>
       <c r="O17" s="11" t="s">
@@ -16758,7 +16762,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[12][17]</v>
       </c>
-      <c r="N18" s="90">
+      <c r="N18" s="86">
         <v>12</v>
       </c>
       <c r="O18" s="11" t="s">
@@ -16884,7 +16888,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[13][17]</v>
       </c>
-      <c r="N19" s="90">
+      <c r="N19" s="86">
         <v>13</v>
       </c>
       <c r="O19" s="11" t="s">
@@ -17010,7 +17014,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[14][17]</v>
       </c>
-      <c r="N20" s="90">
+      <c r="N20" s="86">
         <v>14</v>
       </c>
       <c r="O20" s="11" t="s">
@@ -17136,7 +17140,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[15][17]</v>
       </c>
-      <c r="N21" s="90">
+      <c r="N21" s="86">
         <v>15</v>
       </c>
       <c r="O21" s="11" t="s">
@@ -17262,7 +17266,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[16][17]</v>
       </c>
-      <c r="N22" s="90">
+      <c r="N22" s="86">
         <v>16</v>
       </c>
       <c r="O22" s="11" t="s">
@@ -17388,7 +17392,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[17][17]</v>
       </c>
-      <c r="N23" s="90">
+      <c r="N23" s="86">
         <v>17</v>
       </c>
       <c r="O23" s="11" t="s">
@@ -17514,7 +17518,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[18][17]</v>
       </c>
-      <c r="N24" s="90">
+      <c r="N24" s="86">
         <v>18</v>
       </c>
       <c r="O24" s="11" t="s">
@@ -17640,7 +17644,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[19][17]</v>
       </c>
-      <c r="N25" s="90">
+      <c r="N25" s="86">
         <v>19</v>
       </c>
       <c r="O25" s="11" t="s">
@@ -17766,7 +17770,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[20][17]</v>
       </c>
-      <c r="N26" s="90">
+      <c r="N26" s="86">
         <v>20</v>
       </c>
       <c r="O26" s="11" t="s">
@@ -17892,7 +17896,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[21][17]</v>
       </c>
-      <c r="N27" s="90">
+      <c r="N27" s="86">
         <v>21</v>
       </c>
       <c r="O27" s="11" t="s">
@@ -18018,7 +18022,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[22][17]</v>
       </c>
-      <c r="N28" s="90">
+      <c r="N28" s="86">
         <v>22</v>
       </c>
       <c r="O28" s="11" t="s">
@@ -18144,7 +18148,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[23][17]</v>
       </c>
-      <c r="N29" s="90">
+      <c r="N29" s="86">
         <v>23</v>
       </c>
       <c r="O29" s="11" t="s">
@@ -18270,7 +18274,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[24][17]</v>
       </c>
-      <c r="N30" s="90">
+      <c r="N30" s="86">
         <v>24</v>
       </c>
       <c r="O30" s="11" t="s">
@@ -18396,7 +18400,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[25][17]</v>
       </c>
-      <c r="N31" s="90">
+      <c r="N31" s="86">
         <v>25</v>
       </c>
       <c r="O31" s="11" t="s">
@@ -18522,7 +18526,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[26][17]</v>
       </c>
-      <c r="N32" s="90">
+      <c r="N32" s="86">
         <v>26</v>
       </c>
       <c r="O32" s="11" t="s">
@@ -18648,7 +18652,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[27][17]</v>
       </c>
-      <c r="N33" s="90">
+      <c r="N33" s="86">
         <v>27</v>
       </c>
       <c r="O33" s="11" t="s">
@@ -18774,7 +18778,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[28][17]</v>
       </c>
-      <c r="N34" s="90">
+      <c r="N34" s="86">
         <v>28</v>
       </c>
       <c r="O34" s="11" t="s">
@@ -18900,7 +18904,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[29][17]</v>
       </c>
-      <c r="N35" s="90">
+      <c r="N35" s="86">
         <v>29</v>
       </c>
       <c r="O35" s="11" t="s">
@@ -19026,7 +19030,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[30][17]</v>
       </c>
-      <c r="N36" s="90">
+      <c r="N36" s="86">
         <v>30</v>
       </c>
       <c r="O36" s="11" t="s">
@@ -19152,7 +19156,7 @@
         <f t="shared" si="12"/>
         <v>mp_ac[31][17]</v>
       </c>
-      <c r="N37" s="90">
+      <c r="N37" s="86">
         <v>31</v>
       </c>
       <c r="O37" s="11" t="s">
@@ -19278,7 +19282,7 @@
         <f t="shared" ref="M38:M69" si="27">CONCATENATE("mp_ac[",N38,"][17]")</f>
         <v>mp_ac[32][17]</v>
       </c>
-      <c r="N38" s="90">
+      <c r="N38" s="86">
         <v>32</v>
       </c>
       <c r="O38" s="11" t="s">
@@ -19404,7 +19408,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[33][17]</v>
       </c>
-      <c r="N39" s="90">
+      <c r="N39" s="86">
         <v>33</v>
       </c>
       <c r="O39" s="11" t="s">
@@ -19530,7 +19534,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[34][17]</v>
       </c>
-      <c r="N40" s="90">
+      <c r="N40" s="86">
         <v>34</v>
       </c>
       <c r="O40" s="11" t="s">
@@ -19656,7 +19660,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[35][17]</v>
       </c>
-      <c r="N41" s="90">
+      <c r="N41" s="86">
         <v>35</v>
       </c>
       <c r="O41" s="11" t="s">
@@ -19782,7 +19786,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[36][17]</v>
       </c>
-      <c r="N42" s="90">
+      <c r="N42" s="86">
         <v>36</v>
       </c>
       <c r="O42" s="11" t="s">
@@ -19908,7 +19912,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[37][17]</v>
       </c>
-      <c r="N43" s="90">
+      <c r="N43" s="86">
         <v>37</v>
       </c>
       <c r="O43" s="11" t="s">
@@ -20034,7 +20038,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[38][17]</v>
       </c>
-      <c r="N44" s="90">
+      <c r="N44" s="86">
         <v>38</v>
       </c>
       <c r="O44" s="11" t="s">
@@ -20160,7 +20164,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[39][17]</v>
       </c>
-      <c r="N45" s="90">
+      <c r="N45" s="86">
         <v>39</v>
       </c>
       <c r="O45" s="11" t="s">
@@ -20286,7 +20290,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[40][17]</v>
       </c>
-      <c r="N46" s="90">
+      <c r="N46" s="86">
         <v>40</v>
       </c>
       <c r="O46" s="11" t="s">
@@ -20412,7 +20416,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[41][17]</v>
       </c>
-      <c r="N47" s="90">
+      <c r="N47" s="86">
         <v>41</v>
       </c>
       <c r="O47" s="11" t="s">
@@ -20538,7 +20542,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[42][17]</v>
       </c>
-      <c r="N48" s="90">
+      <c r="N48" s="86">
         <v>42</v>
       </c>
       <c r="O48" s="11" t="s">
@@ -20664,7 +20668,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[43][17]</v>
       </c>
-      <c r="N49" s="90">
+      <c r="N49" s="86">
         <v>43</v>
       </c>
       <c r="O49" s="11" t="s">
@@ -20790,7 +20794,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[44][17]</v>
       </c>
-      <c r="N50" s="90">
+      <c r="N50" s="86">
         <v>44</v>
       </c>
       <c r="O50" s="11" t="s">
@@ -20916,7 +20920,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[45][17]</v>
       </c>
-      <c r="N51" s="90">
+      <c r="N51" s="86">
         <v>45</v>
       </c>
       <c r="O51" s="11" t="s">
@@ -21042,7 +21046,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[46][17]</v>
       </c>
-      <c r="N52" s="90">
+      <c r="N52" s="86">
         <v>46</v>
       </c>
       <c r="O52" s="11" t="s">
@@ -21168,7 +21172,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[47][17]</v>
       </c>
-      <c r="N53" s="90">
+      <c r="N53" s="86">
         <v>47</v>
       </c>
       <c r="O53" s="11" t="s">
@@ -21294,7 +21298,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[48][17]</v>
       </c>
-      <c r="N54" s="90">
+      <c r="N54" s="86">
         <v>48</v>
       </c>
       <c r="O54" s="11" t="s">
@@ -21420,7 +21424,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[49][17]</v>
       </c>
-      <c r="N55" s="90">
+      <c r="N55" s="86">
         <v>49</v>
       </c>
       <c r="O55" s="11" t="s">
@@ -21546,7 +21550,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[50][17]</v>
       </c>
-      <c r="N56" s="90">
+      <c r="N56" s="86">
         <v>50</v>
       </c>
       <c r="O56" s="11" t="s">
@@ -21672,7 +21676,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[51][17]</v>
       </c>
-      <c r="N57" s="90">
+      <c r="N57" s="86">
         <v>51</v>
       </c>
       <c r="O57" s="11" t="s">
@@ -21798,7 +21802,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[52][17]</v>
       </c>
-      <c r="N58" s="90">
+      <c r="N58" s="86">
         <v>52</v>
       </c>
       <c r="O58" s="11" t="s">
@@ -21924,7 +21928,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[53][17]</v>
       </c>
-      <c r="N59" s="90">
+      <c r="N59" s="86">
         <v>53</v>
       </c>
       <c r="O59" s="11" t="s">
@@ -22050,7 +22054,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[54][17]</v>
       </c>
-      <c r="N60" s="90">
+      <c r="N60" s="86">
         <v>54</v>
       </c>
       <c r="O60" s="11" t="s">
@@ -22176,7 +22180,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[55][17]</v>
       </c>
-      <c r="N61" s="90">
+      <c r="N61" s="86">
         <v>55</v>
       </c>
       <c r="O61" s="11" t="s">
@@ -22302,7 +22306,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[56][17]</v>
       </c>
-      <c r="N62" s="90">
+      <c r="N62" s="86">
         <v>56</v>
       </c>
       <c r="O62" s="11" t="s">
@@ -22428,7 +22432,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[57][17]</v>
       </c>
-      <c r="N63" s="90">
+      <c r="N63" s="86">
         <v>57</v>
       </c>
       <c r="O63" s="11" t="s">
@@ -22554,7 +22558,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[58][17]</v>
       </c>
-      <c r="N64" s="90">
+      <c r="N64" s="86">
         <v>58</v>
       </c>
       <c r="O64" s="11" t="s">
@@ -22680,7 +22684,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[59][17]</v>
       </c>
-      <c r="N65" s="90">
+      <c r="N65" s="86">
         <v>59</v>
       </c>
       <c r="O65" s="11" t="s">
@@ -22806,7 +22810,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[60][17]</v>
       </c>
-      <c r="N66" s="90">
+      <c r="N66" s="86">
         <v>60</v>
       </c>
       <c r="O66" s="11" t="s">
@@ -22932,7 +22936,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[61][17]</v>
       </c>
-      <c r="N67" s="90">
+      <c r="N67" s="86">
         <v>61</v>
       </c>
       <c r="O67" s="11" t="s">
@@ -23058,7 +23062,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[62][17]</v>
       </c>
-      <c r="N68" s="90">
+      <c r="N68" s="86">
         <v>62</v>
       </c>
       <c r="O68" s="11" t="s">
@@ -23184,7 +23188,7 @@
         <f t="shared" si="27"/>
         <v>mp_ac[63][17]</v>
       </c>
-      <c r="N69" s="90">
+      <c r="N69" s="86">
         <v>63</v>
       </c>
       <c r="O69" s="11" t="s">
@@ -23310,7 +23314,7 @@
         <f t="shared" ref="M70:M111" si="41">CONCATENATE("mp_ac[",N70,"][17]")</f>
         <v>mp_ac[64][17]</v>
       </c>
-      <c r="N70" s="90">
+      <c r="N70" s="86">
         <v>64</v>
       </c>
       <c r="O70" s="11" t="s">
@@ -23436,7 +23440,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[65][17]</v>
       </c>
-      <c r="N71" s="90">
+      <c r="N71" s="86">
         <v>65</v>
       </c>
       <c r="O71" s="11" t="s">
@@ -23562,7 +23566,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[66][17]</v>
       </c>
-      <c r="N72" s="90">
+      <c r="N72" s="86">
         <v>66</v>
       </c>
       <c r="O72" s="11" t="s">
@@ -23688,7 +23692,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[67][17]</v>
       </c>
-      <c r="N73" s="90">
+      <c r="N73" s="86">
         <v>67</v>
       </c>
       <c r="O73" s="11" t="s">
@@ -23814,7 +23818,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[68][17]</v>
       </c>
-      <c r="N74" s="90">
+      <c r="N74" s="86">
         <v>68</v>
       </c>
       <c r="O74" s="11" t="s">
@@ -23940,7 +23944,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[69][17]</v>
       </c>
-      <c r="N75" s="90">
+      <c r="N75" s="86">
         <v>69</v>
       </c>
       <c r="O75" s="11" t="s">
@@ -24066,7 +24070,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[70][17]</v>
       </c>
-      <c r="N76" s="90">
+      <c r="N76" s="86">
         <v>70</v>
       </c>
       <c r="O76" s="11" t="s">
@@ -24192,7 +24196,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[71][17]</v>
       </c>
-      <c r="N77" s="90">
+      <c r="N77" s="86">
         <v>71</v>
       </c>
       <c r="O77" s="11" t="s">
@@ -24318,7 +24322,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[72][17]</v>
       </c>
-      <c r="N78" s="90">
+      <c r="N78" s="86">
         <v>72</v>
       </c>
       <c r="O78" s="11" t="s">
@@ -24444,7 +24448,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[73][17]</v>
       </c>
-      <c r="N79" s="90">
+      <c r="N79" s="86">
         <v>73</v>
       </c>
       <c r="O79" s="11" t="s">
@@ -24570,7 +24574,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[74][17]</v>
       </c>
-      <c r="N80" s="90">
+      <c r="N80" s="86">
         <v>74</v>
       </c>
       <c r="O80" s="11" t="s">
@@ -24696,7 +24700,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[75][17]</v>
       </c>
-      <c r="N81" s="90">
+      <c r="N81" s="86">
         <v>75</v>
       </c>
       <c r="O81" s="11" t="s">
@@ -24822,7 +24826,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[76][17]</v>
       </c>
-      <c r="N82" s="90">
+      <c r="N82" s="86">
         <v>76</v>
       </c>
       <c r="O82" s="11" t="s">
@@ -24948,7 +24952,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[77][17]</v>
       </c>
-      <c r="N83" s="90">
+      <c r="N83" s="86">
         <v>77</v>
       </c>
       <c r="O83" s="11" t="s">
@@ -25074,7 +25078,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[78][17]</v>
       </c>
-      <c r="N84" s="90">
+      <c r="N84" s="86">
         <v>78</v>
       </c>
       <c r="O84" s="11" t="s">
@@ -25200,7 +25204,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[79][17]</v>
       </c>
-      <c r="N85" s="90">
+      <c r="N85" s="86">
         <v>79</v>
       </c>
       <c r="O85" s="11" t="s">
@@ -25326,7 +25330,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[80][17]</v>
       </c>
-      <c r="N86" s="90">
+      <c r="N86" s="86">
         <v>80</v>
       </c>
       <c r="O86" s="11" t="s">
@@ -25452,7 +25456,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[81][17]</v>
       </c>
-      <c r="N87" s="90">
+      <c r="N87" s="86">
         <v>81</v>
       </c>
       <c r="O87" s="11" t="s">
@@ -25578,7 +25582,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[82][17]</v>
       </c>
-      <c r="N88" s="90">
+      <c r="N88" s="86">
         <v>82</v>
       </c>
       <c r="O88" s="11" t="s">
@@ -25704,7 +25708,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[83][17]</v>
       </c>
-      <c r="N89" s="90">
+      <c r="N89" s="86">
         <v>83</v>
       </c>
       <c r="O89" s="11" t="s">
@@ -25830,7 +25834,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[84][17]</v>
       </c>
-      <c r="N90" s="90">
+      <c r="N90" s="86">
         <v>84</v>
       </c>
       <c r="O90" s="11" t="s">
@@ -25956,7 +25960,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[85][17]</v>
       </c>
-      <c r="N91" s="90">
+      <c r="N91" s="86">
         <v>85</v>
       </c>
       <c r="O91" s="11" t="s">
@@ -26082,7 +26086,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[86][17]</v>
       </c>
-      <c r="N92" s="90">
+      <c r="N92" s="86">
         <v>86</v>
       </c>
       <c r="O92" s="11" t="s">
@@ -26208,7 +26212,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[87][17]</v>
       </c>
-      <c r="N93" s="90">
+      <c r="N93" s="86">
         <v>87</v>
       </c>
       <c r="O93" s="11" t="s">
@@ -26334,7 +26338,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[88][17]</v>
       </c>
-      <c r="N94" s="90">
+      <c r="N94" s="86">
         <v>88</v>
       </c>
       <c r="O94" s="11" t="s">
@@ -26460,7 +26464,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[89][17]</v>
       </c>
-      <c r="N95" s="90">
+      <c r="N95" s="86">
         <v>89</v>
       </c>
       <c r="O95" s="11" t="s">
@@ -26586,7 +26590,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[90][17]</v>
       </c>
-      <c r="N96" s="90">
+      <c r="N96" s="86">
         <v>90</v>
       </c>
       <c r="O96" s="11" t="s">
@@ -26712,7 +26716,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[91][17]</v>
       </c>
-      <c r="N97" s="90">
+      <c r="N97" s="86">
         <v>91</v>
       </c>
       <c r="O97" s="11" t="s">
@@ -26838,7 +26842,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[92][17]</v>
       </c>
-      <c r="N98" s="90">
+      <c r="N98" s="86">
         <v>92</v>
       </c>
       <c r="O98" s="11" t="s">
@@ -26964,7 +26968,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[93][17]</v>
       </c>
-      <c r="N99" s="90">
+      <c r="N99" s="86">
         <v>93</v>
       </c>
       <c r="O99" s="11" t="s">
@@ -27090,7 +27094,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[94][17]</v>
       </c>
-      <c r="N100" s="90">
+      <c r="N100" s="86">
         <v>94</v>
       </c>
       <c r="O100" s="11" t="s">
@@ -27216,7 +27220,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[95][17]</v>
       </c>
-      <c r="N101" s="90">
+      <c r="N101" s="86">
         <v>95</v>
       </c>
       <c r="O101" s="11" t="s">
@@ -27342,7 +27346,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[96][17]</v>
       </c>
-      <c r="N102" s="90">
+      <c r="N102" s="86">
         <v>96</v>
       </c>
       <c r="O102" s="11" t="s">
@@ -27468,7 +27472,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[97][17]</v>
       </c>
-      <c r="N103" s="90">
+      <c r="N103" s="86">
         <v>97</v>
       </c>
       <c r="O103" s="11" t="s">
@@ -27594,7 +27598,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[98][17]</v>
       </c>
-      <c r="N104" s="90">
+      <c r="N104" s="86">
         <v>98</v>
       </c>
       <c r="O104" s="11" t="s">
@@ -27720,7 +27724,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[99][17]</v>
       </c>
-      <c r="N105" s="90">
+      <c r="N105" s="86">
         <v>99</v>
       </c>
       <c r="O105" s="11" t="s">
@@ -27846,7 +27850,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[100][17]</v>
       </c>
-      <c r="N106" s="90">
+      <c r="N106" s="86">
         <v>100</v>
       </c>
       <c r="O106" s="11" t="s">
@@ -27972,7 +27976,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[101][17]</v>
       </c>
-      <c r="N107" s="90">
+      <c r="N107" s="86">
         <v>101</v>
       </c>
       <c r="O107" s="11" t="s">
@@ -28098,7 +28102,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[102][17]</v>
       </c>
-      <c r="N108" s="90">
+      <c r="N108" s="86">
         <v>102</v>
       </c>
       <c r="O108" s="11" t="s">
@@ -28224,7 +28228,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[103][17]</v>
       </c>
-      <c r="N109" s="90">
+      <c r="N109" s="86">
         <v>103</v>
       </c>
       <c r="O109" s="11" t="s">
@@ -28350,7 +28354,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[104][17]</v>
       </c>
-      <c r="N110" s="90">
+      <c r="N110" s="86">
         <v>104</v>
       </c>
       <c r="O110" s="11" t="s">
@@ -28476,7 +28480,7 @@
         <f t="shared" si="41"/>
         <v>mp_ac[105][17]</v>
       </c>
-      <c r="N111" s="90">
+      <c r="N111" s="86">
         <v>105</v>
       </c>
       <c r="O111" s="11" t="s">
@@ -28602,7 +28606,7 @@
         <f t="shared" ref="M112:M143" si="69">CONCATENATE("mp_ac[",N112,"][17]")</f>
         <v>mp_ac[106][17]</v>
       </c>
-      <c r="N112" s="90">
+      <c r="N112" s="86">
         <v>106</v>
       </c>
       <c r="O112" s="11" t="s">
@@ -28728,7 +28732,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[107][17]</v>
       </c>
-      <c r="N113" s="90">
+      <c r="N113" s="86">
         <v>107</v>
       </c>
       <c r="O113" s="11" t="s">
@@ -28854,7 +28858,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[108][17]</v>
       </c>
-      <c r="N114" s="90">
+      <c r="N114" s="86">
         <v>108</v>
       </c>
       <c r="O114" s="11" t="s">
@@ -28980,7 +28984,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[109][17]</v>
       </c>
-      <c r="N115" s="90">
+      <c r="N115" s="86">
         <v>109</v>
       </c>
       <c r="O115" s="11" t="s">
@@ -29106,7 +29110,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[110][17]</v>
       </c>
-      <c r="N116" s="90">
+      <c r="N116" s="86">
         <v>110</v>
       </c>
       <c r="O116" s="11" t="s">
@@ -29232,7 +29236,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[111][17]</v>
       </c>
-      <c r="N117" s="90">
+      <c r="N117" s="86">
         <v>111</v>
       </c>
       <c r="O117" s="11" t="s">
@@ -29358,7 +29362,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[112][17]</v>
       </c>
-      <c r="N118" s="90">
+      <c r="N118" s="86">
         <v>112</v>
       </c>
       <c r="O118" s="11" t="s">
@@ -29484,7 +29488,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[113][17]</v>
       </c>
-      <c r="N119" s="90">
+      <c r="N119" s="86">
         <v>113</v>
       </c>
       <c r="O119" s="11" t="s">
@@ -29610,7 +29614,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[114][17]</v>
       </c>
-      <c r="N120" s="90">
+      <c r="N120" s="86">
         <v>114</v>
       </c>
       <c r="O120" s="11" t="s">
@@ -29736,7 +29740,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[115][17]</v>
       </c>
-      <c r="N121" s="90">
+      <c r="N121" s="86">
         <v>115</v>
       </c>
       <c r="O121" s="11" t="s">
@@ -29862,7 +29866,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[116][17]</v>
       </c>
-      <c r="N122" s="90">
+      <c r="N122" s="86">
         <v>116</v>
       </c>
       <c r="O122" s="11" t="s">
@@ -29988,7 +29992,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[117][17]</v>
       </c>
-      <c r="N123" s="90">
+      <c r="N123" s="86">
         <v>117</v>
       </c>
       <c r="O123" s="11" t="s">
@@ -30114,7 +30118,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[118][17]</v>
       </c>
-      <c r="N124" s="90">
+      <c r="N124" s="86">
         <v>118</v>
       </c>
       <c r="O124" s="11" t="s">
@@ -30240,7 +30244,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[119][17]</v>
       </c>
-      <c r="N125" s="90">
+      <c r="N125" s="86">
         <v>119</v>
       </c>
       <c r="O125" s="11" t="s">
@@ -30366,7 +30370,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[120][17]</v>
       </c>
-      <c r="N126" s="90">
+      <c r="N126" s="86">
         <v>120</v>
       </c>
       <c r="O126" s="11" t="s">
@@ -30492,7 +30496,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[121][17]</v>
       </c>
-      <c r="N127" s="90">
+      <c r="N127" s="86">
         <v>121</v>
       </c>
       <c r="O127" s="11" t="s">
@@ -30618,7 +30622,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[122][17]</v>
       </c>
-      <c r="N128" s="90">
+      <c r="N128" s="86">
         <v>122</v>
       </c>
       <c r="O128" s="11" t="s">
@@ -30744,7 +30748,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[123][17]</v>
       </c>
-      <c r="N129" s="90">
+      <c r="N129" s="86">
         <v>123</v>
       </c>
       <c r="O129" s="11" t="s">
@@ -30870,7 +30874,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[124][17]</v>
       </c>
-      <c r="N130" s="90">
+      <c r="N130" s="86">
         <v>124</v>
       </c>
       <c r="O130" s="11" t="s">
@@ -30996,7 +31000,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[125][17]</v>
       </c>
-      <c r="N131" s="90">
+      <c r="N131" s="86">
         <v>125</v>
       </c>
       <c r="O131" s="11" t="s">
@@ -31122,7 +31126,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[126][17]</v>
       </c>
-      <c r="N132" s="90">
+      <c r="N132" s="86">
         <v>126</v>
       </c>
       <c r="O132" s="11" t="s">
@@ -31248,7 +31252,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[127][17]</v>
       </c>
-      <c r="N133" s="90">
+      <c r="N133" s="86">
         <v>127</v>
       </c>
       <c r="O133" s="11" t="s">
@@ -31374,7 +31378,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[128][17]</v>
       </c>
-      <c r="N134" s="90">
+      <c r="N134" s="86">
         <v>128</v>
       </c>
       <c r="O134" s="11" t="s">
@@ -31500,7 +31504,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[129][17]</v>
       </c>
-      <c r="N135" s="90">
+      <c r="N135" s="86">
         <v>129</v>
       </c>
       <c r="O135" s="11" t="s">
@@ -31626,7 +31630,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[130][17]</v>
       </c>
-      <c r="N136" s="90">
+      <c r="N136" s="86">
         <v>130</v>
       </c>
       <c r="O136" s="11" t="s">
@@ -31752,7 +31756,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[131][17]</v>
       </c>
-      <c r="N137" s="90">
+      <c r="N137" s="86">
         <v>131</v>
       </c>
       <c r="O137" s="11" t="s">
@@ -31878,7 +31882,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[132][17]</v>
       </c>
-      <c r="N138" s="90">
+      <c r="N138" s="86">
         <v>132</v>
       </c>
       <c r="O138" s="11" t="s">
@@ -32004,7 +32008,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[133][17]</v>
       </c>
-      <c r="N139" s="90">
+      <c r="N139" s="86">
         <v>133</v>
       </c>
       <c r="O139" s="11" t="s">
@@ -32130,7 +32134,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[134][17]</v>
       </c>
-      <c r="N140" s="90">
+      <c r="N140" s="86">
         <v>134</v>
       </c>
       <c r="O140" s="11" t="s">
@@ -32256,7 +32260,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[135][17]</v>
       </c>
-      <c r="N141" s="90">
+      <c r="N141" s="86">
         <v>135</v>
       </c>
       <c r="O141" s="11" t="s">
@@ -32382,7 +32386,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[136][17]</v>
       </c>
-      <c r="N142" s="90">
+      <c r="N142" s="86">
         <v>136</v>
       </c>
       <c r="O142" s="11" t="s">
@@ -32508,7 +32512,7 @@
         <f t="shared" si="69"/>
         <v>mp_ac[137][17]</v>
       </c>
-      <c r="N143" s="90">
+      <c r="N143" s="86">
         <v>137</v>
       </c>
       <c r="O143" s="11" t="s">
@@ -32634,7 +32638,7 @@
         <f t="shared" ref="M144:M175" si="83">CONCATENATE("mp_ac[",N144,"][17]")</f>
         <v>mp_ac[138][17]</v>
       </c>
-      <c r="N144" s="90">
+      <c r="N144" s="86">
         <v>138</v>
       </c>
       <c r="O144" s="11" t="s">
@@ -32760,7 +32764,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[139][17]</v>
       </c>
-      <c r="N145" s="90">
+      <c r="N145" s="86">
         <v>139</v>
       </c>
       <c r="O145" s="11" t="s">
@@ -32886,7 +32890,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[140][17]</v>
       </c>
-      <c r="N146" s="90">
+      <c r="N146" s="86">
         <v>140</v>
       </c>
       <c r="O146" s="11" t="s">
@@ -33012,7 +33016,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[141][17]</v>
       </c>
-      <c r="N147" s="90">
+      <c r="N147" s="86">
         <v>141</v>
       </c>
       <c r="O147" s="11" t="s">
@@ -33138,7 +33142,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[142][17]</v>
       </c>
-      <c r="N148" s="90">
+      <c r="N148" s="86">
         <v>142</v>
       </c>
       <c r="O148" s="11" t="s">
@@ -33264,7 +33268,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[143][17]</v>
       </c>
-      <c r="N149" s="90">
+      <c r="N149" s="86">
         <v>143</v>
       </c>
       <c r="O149" s="11" t="s">
@@ -33390,7 +33394,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[144][17]</v>
       </c>
-      <c r="N150" s="90">
+      <c r="N150" s="86">
         <v>144</v>
       </c>
       <c r="O150" s="11" t="s">
@@ -33516,7 +33520,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[145][17]</v>
       </c>
-      <c r="N151" s="90">
+      <c r="N151" s="86">
         <v>145</v>
       </c>
       <c r="O151" s="11" t="s">
@@ -33642,7 +33646,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[146][17]</v>
       </c>
-      <c r="N152" s="90">
+      <c r="N152" s="86">
         <v>146</v>
       </c>
       <c r="O152" s="11" t="s">
@@ -33768,7 +33772,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[147][17]</v>
       </c>
-      <c r="N153" s="90">
+      <c r="N153" s="86">
         <v>147</v>
       </c>
       <c r="O153" s="11" t="s">
@@ -33894,7 +33898,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[148][17]</v>
       </c>
-      <c r="N154" s="90">
+      <c r="N154" s="86">
         <v>148</v>
       </c>
       <c r="O154" s="11" t="s">
@@ -34020,7 +34024,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[149][17]</v>
       </c>
-      <c r="N155" s="90">
+      <c r="N155" s="86">
         <v>149</v>
       </c>
       <c r="O155" s="11" t="s">
@@ -34146,7 +34150,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[150][17]</v>
       </c>
-      <c r="N156" s="90">
+      <c r="N156" s="86">
         <v>150</v>
       </c>
       <c r="O156" s="11" t="s">
@@ -34272,7 +34276,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[151][17]</v>
       </c>
-      <c r="N157" s="90">
+      <c r="N157" s="86">
         <v>151</v>
       </c>
       <c r="O157" s="11" t="s">
@@ -34398,7 +34402,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[152][17]</v>
       </c>
-      <c r="N158" s="90">
+      <c r="N158" s="86">
         <v>152</v>
       </c>
       <c r="O158" s="11" t="s">
@@ -34524,7 +34528,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[153][17]</v>
       </c>
-      <c r="N159" s="90">
+      <c r="N159" s="86">
         <v>153</v>
       </c>
       <c r="O159" s="11" t="s">
@@ -34650,7 +34654,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[154][17]</v>
       </c>
-      <c r="N160" s="90">
+      <c r="N160" s="86">
         <v>154</v>
       </c>
       <c r="O160" s="11" t="s">
@@ -34776,7 +34780,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[155][17]</v>
       </c>
-      <c r="N161" s="90">
+      <c r="N161" s="86">
         <v>155</v>
       </c>
       <c r="O161" s="11" t="s">
@@ -34902,7 +34906,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[156][17]</v>
       </c>
-      <c r="N162" s="90">
+      <c r="N162" s="86">
         <v>156</v>
       </c>
       <c r="O162" s="11" t="s">
@@ -35028,7 +35032,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[157][17]</v>
       </c>
-      <c r="N163" s="90">
+      <c r="N163" s="86">
         <v>157</v>
       </c>
       <c r="O163" s="11" t="s">
@@ -35154,7 +35158,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[158][17]</v>
       </c>
-      <c r="N164" s="90">
+      <c r="N164" s="86">
         <v>158</v>
       </c>
       <c r="O164" s="11" t="s">
@@ -35280,7 +35284,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[159][17]</v>
       </c>
-      <c r="N165" s="90">
+      <c r="N165" s="86">
         <v>159</v>
       </c>
       <c r="O165" s="11" t="s">
@@ -35406,7 +35410,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[160][17]</v>
       </c>
-      <c r="N166" s="90">
+      <c r="N166" s="86">
         <v>160</v>
       </c>
       <c r="O166" s="11" t="s">
@@ -35532,7 +35536,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[161][17]</v>
       </c>
-      <c r="N167" s="90">
+      <c r="N167" s="86">
         <v>161</v>
       </c>
       <c r="O167" s="11" t="s">
@@ -35658,7 +35662,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[162][17]</v>
       </c>
-      <c r="N168" s="90">
+      <c r="N168" s="86">
         <v>162</v>
       </c>
       <c r="O168" s="11" t="s">
@@ -35784,7 +35788,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[163][17]</v>
       </c>
-      <c r="N169" s="90">
+      <c r="N169" s="86">
         <v>163</v>
       </c>
       <c r="O169" s="11" t="s">
@@ -35910,7 +35914,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[164][17]</v>
       </c>
-      <c r="N170" s="90">
+      <c r="N170" s="86">
         <v>164</v>
       </c>
       <c r="O170" s="11" t="s">
@@ -36036,7 +36040,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[165][17]</v>
       </c>
-      <c r="N171" s="90">
+      <c r="N171" s="86">
         <v>165</v>
       </c>
       <c r="O171" s="11" t="s">
@@ -36162,7 +36166,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[166][17]</v>
       </c>
-      <c r="N172" s="90">
+      <c r="N172" s="86">
         <v>166</v>
       </c>
       <c r="O172" s="11" t="s">
@@ -36288,7 +36292,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[167][17]</v>
       </c>
-      <c r="N173" s="90">
+      <c r="N173" s="86">
         <v>167</v>
       </c>
       <c r="O173" s="11" t="s">
@@ -36414,7 +36418,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[168][17]</v>
       </c>
-      <c r="N174" s="90">
+      <c r="N174" s="86">
         <v>168</v>
       </c>
       <c r="O174" s="11" t="s">
@@ -36540,7 +36544,7 @@
         <f t="shared" si="83"/>
         <v>mp_ac[169][17]</v>
       </c>
-      <c r="N175" s="90">
+      <c r="N175" s="86">
         <v>169</v>
       </c>
       <c r="O175" s="11" t="s">
@@ -36666,7 +36670,7 @@
         <f t="shared" ref="M176:M201" si="97">CONCATENATE("mp_ac[",N176,"][17]")</f>
         <v>mp_ac[170][17]</v>
       </c>
-      <c r="N176" s="90">
+      <c r="N176" s="86">
         <v>170</v>
       </c>
       <c r="O176" s="11" t="s">
@@ -36792,7 +36796,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[171][17]</v>
       </c>
-      <c r="N177" s="90">
+      <c r="N177" s="86">
         <v>171</v>
       </c>
       <c r="O177" s="11" t="s">
@@ -36918,7 +36922,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[172][17]</v>
       </c>
-      <c r="N178" s="90">
+      <c r="N178" s="86">
         <v>172</v>
       </c>
       <c r="O178" s="11" t="s">
@@ -37044,7 +37048,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[173][17]</v>
       </c>
-      <c r="N179" s="90">
+      <c r="N179" s="86">
         <v>173</v>
       </c>
       <c r="O179" s="11" t="s">
@@ -37170,7 +37174,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[174][17]</v>
       </c>
-      <c r="N180" s="90">
+      <c r="N180" s="86">
         <v>174</v>
       </c>
       <c r="O180" s="11" t="s">
@@ -37296,7 +37300,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[175][17]</v>
       </c>
-      <c r="N181" s="90">
+      <c r="N181" s="86">
         <v>175</v>
       </c>
       <c r="O181" s="11" t="s">
@@ -37422,7 +37426,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[176][17]</v>
       </c>
-      <c r="N182" s="90">
+      <c r="N182" s="86">
         <v>176</v>
       </c>
       <c r="O182" s="11" t="s">
@@ -37548,7 +37552,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[177][17]</v>
       </c>
-      <c r="N183" s="90">
+      <c r="N183" s="86">
         <v>177</v>
       </c>
       <c r="O183" s="11" t="s">
@@ -37674,7 +37678,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[178][17]</v>
       </c>
-      <c r="N184" s="90">
+      <c r="N184" s="86">
         <v>178</v>
       </c>
       <c r="O184" s="11" t="s">
@@ -37800,7 +37804,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[179][17]</v>
       </c>
-      <c r="N185" s="90">
+      <c r="N185" s="86">
         <v>179</v>
       </c>
       <c r="O185" s="11" t="s">
@@ -37926,7 +37930,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[180][17]</v>
       </c>
-      <c r="N186" s="90">
+      <c r="N186" s="86">
         <v>180</v>
       </c>
       <c r="O186" s="11" t="s">
@@ -38052,7 +38056,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[181][17]</v>
       </c>
-      <c r="N187" s="90">
+      <c r="N187" s="86">
         <v>181</v>
       </c>
       <c r="O187" s="11" t="s">
@@ -38178,7 +38182,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[182][17]</v>
       </c>
-      <c r="N188" s="90">
+      <c r="N188" s="86">
         <v>182</v>
       </c>
       <c r="O188" s="11" t="s">
@@ -38304,7 +38308,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[183][17]</v>
       </c>
-      <c r="N189" s="90">
+      <c r="N189" s="86">
         <v>183</v>
       </c>
       <c r="O189" s="11" t="s">
@@ -38430,7 +38434,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[184][17]</v>
       </c>
-      <c r="N190" s="90">
+      <c r="N190" s="86">
         <v>184</v>
       </c>
       <c r="O190" s="11" t="s">
@@ -38556,7 +38560,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[185][17]</v>
       </c>
-      <c r="N191" s="90">
+      <c r="N191" s="86">
         <v>185</v>
       </c>
       <c r="O191" s="11" t="s">
@@ -38682,7 +38686,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[186][17]</v>
       </c>
-      <c r="N192" s="90">
+      <c r="N192" s="86">
         <v>186</v>
       </c>
       <c r="O192" s="11" t="s">
@@ -38808,7 +38812,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[187][17]</v>
       </c>
-      <c r="N193" s="90">
+      <c r="N193" s="86">
         <v>187</v>
       </c>
       <c r="O193" s="11" t="s">
@@ -38934,7 +38938,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[188][17]</v>
       </c>
-      <c r="N194" s="90">
+      <c r="N194" s="86">
         <v>188</v>
       </c>
       <c r="O194" s="11" t="s">
@@ -39060,7 +39064,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[189][17]</v>
       </c>
-      <c r="N195" s="90">
+      <c r="N195" s="86">
         <v>189</v>
       </c>
       <c r="O195" s="11" t="s">
@@ -39186,7 +39190,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[190][17]</v>
       </c>
-      <c r="N196" s="90">
+      <c r="N196" s="86">
         <v>190</v>
       </c>
       <c r="O196" s="11" t="s">
@@ -39312,7 +39316,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[191][17]</v>
       </c>
-      <c r="N197" s="90">
+      <c r="N197" s="86">
         <v>191</v>
       </c>
       <c r="O197" s="11" t="s">
@@ -39438,7 +39442,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[192][17]</v>
       </c>
-      <c r="N198" s="90">
+      <c r="N198" s="86">
         <v>192</v>
       </c>
       <c r="O198" s="11" t="s">
@@ -39564,7 +39568,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[193][17]</v>
       </c>
-      <c r="N199" s="90">
+      <c r="N199" s="86">
         <v>193</v>
       </c>
       <c r="O199" s="11" t="s">
@@ -39690,7 +39694,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[194][17]</v>
       </c>
-      <c r="N200" s="90">
+      <c r="N200" s="86">
         <v>194</v>
       </c>
       <c r="O200" s="11" t="s">
@@ -39816,7 +39820,7 @@
         <f t="shared" si="97"/>
         <v>mp_ac[195][17]</v>
       </c>
-      <c r="N201" s="90">
+      <c r="N201" s="86">
         <v>195</v>
       </c>
       <c r="O201" s="11" t="s">
@@ -39893,70 +39897,70 @@
       <c r="G202" s="65"/>
       <c r="H202" s="65"/>
       <c r="I202" s="65"/>
-      <c r="J202" s="87" t="s">
+      <c r="J202" s="91" t="s">
         <v>1338</v>
       </c>
-      <c r="K202" s="87"/>
-      <c r="L202" s="87"/>
+      <c r="K202" s="91"/>
+      <c r="L202" s="91"/>
       <c r="M202" s="66" t="str">
         <f t="shared" ref="M202:M207" si="112">CONCATENATE("mp_ac[",N202,"][3]")</f>
         <v>mp_ac[196][3]</v>
       </c>
-      <c r="N202" s="90">
+      <c r="N202" s="86">
         <v>196</v>
       </c>
-      <c r="O202" s="91" t="s">
+      <c r="O202" s="87" t="s">
         <v>1307</v>
       </c>
-      <c r="P202" s="91" t="s">
+      <c r="P202" s="87" t="s">
         <v>1307</v>
       </c>
-      <c r="Q202" s="92" t="s">
+      <c r="Q202" s="88" t="s">
         <v>1315</v>
       </c>
-      <c r="R202" s="93" t="s">
+      <c r="R202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="S202" s="93" t="s">
+      <c r="S202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="T202" s="93" t="s">
+      <c r="T202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="U202" s="93" t="s">
+      <c r="U202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="V202" s="93" t="s">
+      <c r="V202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="W202" s="93" t="s">
+      <c r="W202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="X202" s="93" t="s">
+      <c r="X202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Y202" s="93" t="s">
+      <c r="Y202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Z202" s="93" t="s">
+      <c r="Z202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AA202" s="93" t="s">
+      <c r="AA202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AB202" s="93" t="s">
+      <c r="AB202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AC202" s="93" t="s">
+      <c r="AC202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AD202" s="93" t="s">
+      <c r="AD202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AE202" s="93" t="s">
+      <c r="AE202" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AF202" s="93" t="s">
+      <c r="AF202" s="89" t="s">
         <v>495</v>
       </c>
       <c r="AH202" s="6" t="s">
@@ -39975,68 +39979,68 @@
       <c r="G203" s="65"/>
       <c r="H203" s="65"/>
       <c r="I203" s="65"/>
-      <c r="J203" s="87"/>
-      <c r="K203" s="87"/>
-      <c r="L203" s="87"/>
+      <c r="J203" s="91"/>
+      <c r="K203" s="91"/>
+      <c r="L203" s="91"/>
       <c r="M203" s="66" t="str">
         <f t="shared" si="112"/>
         <v>mp_ac[197][3]</v>
       </c>
-      <c r="N203" s="90">
+      <c r="N203" s="86">
         <v>197</v>
       </c>
-      <c r="O203" s="91" t="s">
+      <c r="O203" s="87" t="s">
         <v>1308</v>
       </c>
-      <c r="P203" s="91" t="s">
+      <c r="P203" s="87" t="s">
         <v>1308</v>
       </c>
-      <c r="Q203" s="92" t="s">
+      <c r="Q203" s="88" t="s">
         <v>1316</v>
       </c>
-      <c r="R203" s="93" t="s">
+      <c r="R203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="S203" s="93" t="s">
+      <c r="S203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="T203" s="93" t="s">
+      <c r="T203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="U203" s="93" t="s">
+      <c r="U203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="V203" s="93" t="s">
+      <c r="V203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="W203" s="93" t="s">
+      <c r="W203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="X203" s="93" t="s">
+      <c r="X203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Y203" s="93" t="s">
+      <c r="Y203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Z203" s="93" t="s">
+      <c r="Z203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AA203" s="93" t="s">
+      <c r="AA203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AB203" s="93" t="s">
+      <c r="AB203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AC203" s="93" t="s">
+      <c r="AC203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AD203" s="93" t="s">
+      <c r="AD203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AE203" s="93" t="s">
+      <c r="AE203" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AF203" s="93" t="s">
+      <c r="AF203" s="89" t="s">
         <v>495</v>
       </c>
       <c r="AH203" s="6" t="s">
@@ -40055,68 +40059,68 @@
       <c r="G204" s="65"/>
       <c r="H204" s="65"/>
       <c r="I204" s="65"/>
-      <c r="J204" s="87"/>
-      <c r="K204" s="87"/>
-      <c r="L204" s="87"/>
+      <c r="J204" s="91"/>
+      <c r="K204" s="91"/>
+      <c r="L204" s="91"/>
       <c r="M204" s="66" t="str">
         <f t="shared" si="112"/>
         <v>mp_ac[198][3]</v>
       </c>
-      <c r="N204" s="90">
+      <c r="N204" s="86">
         <v>198</v>
       </c>
-      <c r="O204" s="91" t="s">
+      <c r="O204" s="87" t="s">
         <v>1309</v>
       </c>
-      <c r="P204" s="91" t="s">
+      <c r="P204" s="87" t="s">
         <v>1309</v>
       </c>
-      <c r="Q204" s="92" t="s">
+      <c r="Q204" s="88" t="s">
         <v>1317</v>
       </c>
-      <c r="R204" s="93" t="s">
+      <c r="R204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="S204" s="93" t="s">
+      <c r="S204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="T204" s="93" t="s">
+      <c r="T204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="U204" s="93" t="s">
+      <c r="U204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="V204" s="93" t="s">
+      <c r="V204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="W204" s="93" t="s">
+      <c r="W204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="X204" s="93" t="s">
+      <c r="X204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Y204" s="93" t="s">
+      <c r="Y204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Z204" s="93" t="s">
+      <c r="Z204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AA204" s="93" t="s">
+      <c r="AA204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AB204" s="93" t="s">
+      <c r="AB204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AC204" s="93" t="s">
+      <c r="AC204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AD204" s="93" t="s">
+      <c r="AD204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AE204" s="93" t="s">
+      <c r="AE204" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AF204" s="93" t="s">
+      <c r="AF204" s="89" t="s">
         <v>495</v>
       </c>
       <c r="AH204" s="6" t="s">
@@ -40135,68 +40139,68 @@
       <c r="G205" s="65"/>
       <c r="H205" s="65"/>
       <c r="I205" s="65"/>
-      <c r="J205" s="87"/>
-      <c r="K205" s="87"/>
-      <c r="L205" s="87"/>
+      <c r="J205" s="91"/>
+      <c r="K205" s="91"/>
+      <c r="L205" s="91"/>
       <c r="M205" s="66" t="str">
         <f t="shared" si="112"/>
         <v>mp_ac[199][3]</v>
       </c>
-      <c r="N205" s="90">
+      <c r="N205" s="86">
         <v>199</v>
       </c>
-      <c r="O205" s="91" t="s">
+      <c r="O205" s="87" t="s">
         <v>1310</v>
       </c>
-      <c r="P205" s="91" t="s">
+      <c r="P205" s="87" t="s">
         <v>1310</v>
       </c>
-      <c r="Q205" s="92" t="s">
+      <c r="Q205" s="88" t="s">
         <v>1318</v>
       </c>
-      <c r="R205" s="93" t="s">
+      <c r="R205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="S205" s="93" t="s">
+      <c r="S205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="T205" s="93" t="s">
+      <c r="T205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="U205" s="93" t="s">
+      <c r="U205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="V205" s="93" t="s">
+      <c r="V205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="W205" s="93" t="s">
+      <c r="W205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="X205" s="93" t="s">
+      <c r="X205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Y205" s="93" t="s">
+      <c r="Y205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Z205" s="93" t="s">
+      <c r="Z205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AA205" s="93" t="s">
+      <c r="AA205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AB205" s="93" t="s">
+      <c r="AB205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AC205" s="93" t="s">
+      <c r="AC205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AD205" s="93" t="s">
+      <c r="AD205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AE205" s="93" t="s">
+      <c r="AE205" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AF205" s="93" t="s">
+      <c r="AF205" s="89" t="s">
         <v>495</v>
       </c>
       <c r="AH205" s="6" t="s">
@@ -40215,68 +40219,68 @@
       <c r="G206" s="65"/>
       <c r="H206" s="65"/>
       <c r="I206" s="65"/>
-      <c r="J206" s="87"/>
-      <c r="K206" s="87"/>
-      <c r="L206" s="87"/>
+      <c r="J206" s="91"/>
+      <c r="K206" s="91"/>
+      <c r="L206" s="91"/>
       <c r="M206" s="66" t="str">
         <f t="shared" si="112"/>
         <v>mp_ac[200][3]</v>
       </c>
-      <c r="N206" s="90">
+      <c r="N206" s="86">
         <v>200</v>
       </c>
-      <c r="O206" s="91" t="s">
+      <c r="O206" s="87" t="s">
         <v>1311</v>
       </c>
-      <c r="P206" s="91" t="s">
+      <c r="P206" s="87" t="s">
         <v>1311</v>
       </c>
-      <c r="Q206" s="92" t="s">
+      <c r="Q206" s="88" t="s">
         <v>1319</v>
       </c>
-      <c r="R206" s="93" t="s">
+      <c r="R206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="S206" s="93" t="s">
+      <c r="S206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="T206" s="93" t="s">
+      <c r="T206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="U206" s="93" t="s">
+      <c r="U206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="V206" s="93" t="s">
+      <c r="V206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="W206" s="93" t="s">
+      <c r="W206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="X206" s="93" t="s">
+      <c r="X206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Y206" s="93" t="s">
+      <c r="Y206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Z206" s="93" t="s">
+      <c r="Z206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AA206" s="93" t="s">
+      <c r="AA206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AB206" s="93" t="s">
+      <c r="AB206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AC206" s="93" t="s">
+      <c r="AC206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AD206" s="93" t="s">
+      <c r="AD206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AE206" s="93" t="s">
+      <c r="AE206" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AF206" s="93" t="s">
+      <c r="AF206" s="89" t="s">
         <v>495</v>
       </c>
       <c r="AH206" s="6" t="s">
@@ -40295,68 +40299,68 @@
       <c r="G207" s="65"/>
       <c r="H207" s="65"/>
       <c r="I207" s="65"/>
-      <c r="J207" s="88"/>
-      <c r="K207" s="88"/>
-      <c r="L207" s="88"/>
+      <c r="J207" s="92"/>
+      <c r="K207" s="92"/>
+      <c r="L207" s="92"/>
       <c r="M207" s="67" t="str">
         <f t="shared" si="112"/>
         <v>mp_ac[201][3]</v>
       </c>
-      <c r="N207" s="90">
+      <c r="N207" s="86">
         <v>201</v>
       </c>
-      <c r="O207" s="91" t="s">
+      <c r="O207" s="87" t="s">
         <v>1312</v>
       </c>
-      <c r="P207" s="91" t="s">
+      <c r="P207" s="87" t="s">
         <v>1312</v>
       </c>
-      <c r="Q207" s="92" t="s">
+      <c r="Q207" s="88" t="s">
         <v>1320</v>
       </c>
-      <c r="R207" s="93" t="s">
+      <c r="R207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="S207" s="93" t="s">
+      <c r="S207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="T207" s="93" t="s">
+      <c r="T207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="U207" s="93" t="s">
+      <c r="U207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="V207" s="93" t="s">
+      <c r="V207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="W207" s="93" t="s">
+      <c r="W207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="X207" s="93" t="s">
+      <c r="X207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Y207" s="93" t="s">
+      <c r="Y207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="Z207" s="93" t="s">
+      <c r="Z207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AA207" s="93" t="s">
+      <c r="AA207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AB207" s="93" t="s">
+      <c r="AB207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AC207" s="93" t="s">
+      <c r="AC207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AD207" s="93" t="s">
+      <c r="AD207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AE207" s="93" t="s">
+      <c r="AE207" s="89" t="s">
         <v>495</v>
       </c>
-      <c r="AF207" s="93" t="s">
+      <c r="AF207" s="89" t="s">
         <v>495</v>
       </c>
       <c r="AH207" s="6" t="s">
@@ -40400,16 +40404,16 @@
         <f t="shared" ref="M208:M261" si="119">CONCATENATE("mp_ac[",N208,"][17]")</f>
         <v>mp_ac[202][17]</v>
       </c>
-      <c r="N208" s="90">
+      <c r="N208" s="86">
         <v>202</v>
       </c>
-      <c r="O208" s="91" t="s">
+      <c r="O208" s="87" t="s">
         <v>1313</v>
       </c>
-      <c r="P208" s="91" t="s">
+      <c r="P208" s="87" t="s">
         <v>1313</v>
       </c>
-      <c r="Q208" s="92" t="s">
+      <c r="Q208" s="88" t="s">
         <v>1321</v>
       </c>
       <c r="R208" s="37" t="s">
@@ -40494,16 +40498,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[203][17]</v>
       </c>
-      <c r="N209" s="90">
+      <c r="N209" s="86">
         <v>203</v>
       </c>
-      <c r="O209" s="91" t="s">
+      <c r="O209" s="87" t="s">
         <v>1314</v>
       </c>
-      <c r="P209" s="91" t="s">
+      <c r="P209" s="87" t="s">
         <v>1314</v>
       </c>
-      <c r="Q209" s="92" t="s">
+      <c r="Q209" s="88" t="s">
         <v>1322</v>
       </c>
       <c r="R209" s="37" t="s">
@@ -40588,16 +40592,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[204][17]</v>
       </c>
-      <c r="N210" s="90">
+      <c r="N210" s="86">
         <v>204</v>
       </c>
-      <c r="O210" s="91" t="s">
+      <c r="O210" s="87" t="s">
         <v>1292</v>
       </c>
-      <c r="P210" s="91" t="s">
+      <c r="P210" s="87" t="s">
         <v>1292</v>
       </c>
-      <c r="Q210" s="92" t="s">
+      <c r="Q210" s="88" t="s">
         <v>1322</v>
       </c>
       <c r="R210" s="37" t="s">
@@ -40682,16 +40686,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[205][17]</v>
       </c>
-      <c r="N211" s="90">
+      <c r="N211" s="86">
         <v>205</v>
       </c>
-      <c r="O211" s="91" t="s">
+      <c r="O211" s="87" t="s">
         <v>1293</v>
       </c>
-      <c r="P211" s="91" t="s">
+      <c r="P211" s="87" t="s">
         <v>1293</v>
       </c>
-      <c r="Q211" s="92" t="s">
+      <c r="Q211" s="88" t="s">
         <v>1323</v>
       </c>
       <c r="R211" s="37" t="s">
@@ -40776,16 +40780,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[206][17]</v>
       </c>
-      <c r="N212" s="90">
+      <c r="N212" s="86">
         <v>206</v>
       </c>
-      <c r="O212" s="91" t="s">
+      <c r="O212" s="87" t="s">
         <v>1294</v>
       </c>
-      <c r="P212" s="91" t="s">
+      <c r="P212" s="87" t="s">
         <v>1294</v>
       </c>
-      <c r="Q212" s="92" t="s">
+      <c r="Q212" s="88" t="s">
         <v>1324</v>
       </c>
       <c r="R212" s="37" t="s">
@@ -40870,16 +40874,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[207][17]</v>
       </c>
-      <c r="N213" s="90">
+      <c r="N213" s="86">
         <v>207</v>
       </c>
-      <c r="O213" s="91" t="s">
+      <c r="O213" s="87" t="s">
         <v>1295</v>
       </c>
-      <c r="P213" s="91" t="s">
+      <c r="P213" s="87" t="s">
         <v>1295</v>
       </c>
-      <c r="Q213" s="92" t="s">
+      <c r="Q213" s="88" t="s">
         <v>1324</v>
       </c>
       <c r="R213" s="37" t="s">
@@ -40964,16 +40968,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[208][17]</v>
       </c>
-      <c r="N214" s="90">
+      <c r="N214" s="86">
         <v>208</v>
       </c>
-      <c r="O214" s="91" t="s">
+      <c r="O214" s="87" t="s">
         <v>1296</v>
       </c>
-      <c r="P214" s="91" t="s">
+      <c r="P214" s="87" t="s">
         <v>1296</v>
       </c>
-      <c r="Q214" s="92" t="s">
+      <c r="Q214" s="88" t="s">
         <v>1325</v>
       </c>
       <c r="R214" s="37" t="s">
@@ -41058,16 +41062,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[209][17]</v>
       </c>
-      <c r="N215" s="90">
+      <c r="N215" s="86">
         <v>209</v>
       </c>
-      <c r="O215" s="91" t="s">
+      <c r="O215" s="87" t="s">
         <v>1297</v>
       </c>
-      <c r="P215" s="91" t="s">
+      <c r="P215" s="87" t="s">
         <v>1297</v>
       </c>
-      <c r="Q215" s="92" t="s">
+      <c r="Q215" s="88" t="s">
         <v>1325</v>
       </c>
       <c r="R215" s="37" t="s">
@@ -41152,16 +41156,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[210][17]</v>
       </c>
-      <c r="N216" s="90">
+      <c r="N216" s="86">
         <v>210</v>
       </c>
-      <c r="O216" s="91" t="s">
+      <c r="O216" s="87" t="s">
         <v>1298</v>
       </c>
-      <c r="P216" s="91" t="s">
+      <c r="P216" s="87" t="s">
         <v>1298</v>
       </c>
-      <c r="Q216" s="92" t="s">
+      <c r="Q216" s="88" t="s">
         <v>1325</v>
       </c>
       <c r="R216" s="37" t="s">
@@ -41246,16 +41250,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[211][17]</v>
       </c>
-      <c r="N217" s="90">
+      <c r="N217" s="86">
         <v>211</v>
       </c>
-      <c r="O217" s="91" t="s">
+      <c r="O217" s="87" t="s">
         <v>1299</v>
       </c>
-      <c r="P217" s="91" t="s">
+      <c r="P217" s="87" t="s">
         <v>1299</v>
       </c>
-      <c r="Q217" s="92" t="s">
+      <c r="Q217" s="88" t="s">
         <v>1326</v>
       </c>
       <c r="R217" s="37" t="s">
@@ -41340,16 +41344,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[212][17]</v>
       </c>
-      <c r="N218" s="90">
+      <c r="N218" s="86">
         <v>212</v>
       </c>
-      <c r="O218" s="91" t="s">
+      <c r="O218" s="87" t="s">
         <v>1300</v>
       </c>
-      <c r="P218" s="91" t="s">
+      <c r="P218" s="87" t="s">
         <v>1300</v>
       </c>
-      <c r="Q218" s="92" t="s">
+      <c r="Q218" s="88" t="s">
         <v>1326</v>
       </c>
       <c r="R218" s="37" t="s">
@@ -41434,16 +41438,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[213][17]</v>
       </c>
-      <c r="N219" s="90">
+      <c r="N219" s="86">
         <v>213</v>
       </c>
-      <c r="O219" s="91" t="s">
+      <c r="O219" s="87" t="s">
         <v>1298</v>
       </c>
-      <c r="P219" s="91" t="s">
+      <c r="P219" s="87" t="s">
         <v>1298</v>
       </c>
-      <c r="Q219" s="92" t="s">
+      <c r="Q219" s="88" t="s">
         <v>1327</v>
       </c>
       <c r="R219" s="37" t="s">
@@ -41528,16 +41532,16 @@
         <f t="shared" ref="M220:M225" si="127">CONCATENATE("mp_ac[",N220,"][17]")</f>
         <v>mp_ac[214][17]</v>
       </c>
-      <c r="N220" s="90">
+      <c r="N220" s="86">
         <v>214</v>
       </c>
-      <c r="O220" s="91" t="s">
+      <c r="O220" s="87" t="s">
         <v>1556</v>
       </c>
-      <c r="P220" s="91" t="s">
+      <c r="P220" s="87" t="s">
         <v>1556</v>
       </c>
-      <c r="Q220" s="92" t="s">
+      <c r="Q220" s="88" t="s">
         <v>1592</v>
       </c>
       <c r="R220" s="37" t="s">
@@ -41622,16 +41626,16 @@
         <f t="shared" si="127"/>
         <v>mp_ac[215][17]</v>
       </c>
-      <c r="N221" s="90">
+      <c r="N221" s="86">
         <v>215</v>
       </c>
-      <c r="O221" s="91" t="s">
+      <c r="O221" s="87" t="s">
         <v>1557</v>
       </c>
-      <c r="P221" s="91" t="s">
+      <c r="P221" s="87" t="s">
         <v>1557</v>
       </c>
-      <c r="Q221" s="92" t="s">
+      <c r="Q221" s="88" t="s">
         <v>1592</v>
       </c>
       <c r="R221" s="37" t="s">
@@ -41716,16 +41720,16 @@
         <f t="shared" si="127"/>
         <v>mp_ac[216][17]</v>
       </c>
-      <c r="N222" s="90">
+      <c r="N222" s="86">
         <v>216</v>
       </c>
-      <c r="O222" s="91" t="s">
+      <c r="O222" s="87" t="s">
         <v>1558</v>
       </c>
-      <c r="P222" s="91" t="s">
+      <c r="P222" s="87" t="s">
         <v>1558</v>
       </c>
-      <c r="Q222" s="92" t="s">
+      <c r="Q222" s="88" t="s">
         <v>1592</v>
       </c>
       <c r="R222" s="37" t="s">
@@ -41810,16 +41814,16 @@
         <f t="shared" si="127"/>
         <v>mp_ac[217][17]</v>
       </c>
-      <c r="N223" s="90">
+      <c r="N223" s="86">
         <v>217</v>
       </c>
-      <c r="O223" s="91" t="s">
+      <c r="O223" s="87" t="s">
         <v>1559</v>
       </c>
-      <c r="P223" s="91" t="s">
+      <c r="P223" s="87" t="s">
         <v>1559</v>
       </c>
-      <c r="Q223" s="92" t="s">
+      <c r="Q223" s="88" t="s">
         <v>1593</v>
       </c>
       <c r="R223" s="37" t="s">
@@ -41904,16 +41908,16 @@
         <f t="shared" si="127"/>
         <v>mp_ac[218][17]</v>
       </c>
-      <c r="N224" s="90">
+      <c r="N224" s="86">
         <v>218</v>
       </c>
-      <c r="O224" s="91" t="s">
+      <c r="O224" s="87" t="s">
         <v>1560</v>
       </c>
-      <c r="P224" s="91" t="s">
+      <c r="P224" s="87" t="s">
         <v>1560</v>
       </c>
-      <c r="Q224" s="92" t="s">
+      <c r="Q224" s="88" t="s">
         <v>1593</v>
       </c>
       <c r="R224" s="37" t="s">
@@ -41998,16 +42002,16 @@
         <f t="shared" si="127"/>
         <v>mp_ac[219][17]</v>
       </c>
-      <c r="N225" s="90">
+      <c r="N225" s="86">
         <v>219</v>
       </c>
-      <c r="O225" s="91" t="s">
+      <c r="O225" s="87" t="s">
         <v>1561</v>
       </c>
-      <c r="P225" s="91" t="s">
+      <c r="P225" s="87" t="s">
         <v>1561</v>
       </c>
-      <c r="Q225" s="92" t="s">
+      <c r="Q225" s="88" t="s">
         <v>1593</v>
       </c>
       <c r="R225" s="37" t="s">
@@ -42092,16 +42096,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[220][17]</v>
       </c>
-      <c r="N226" s="90">
+      <c r="N226" s="86">
         <v>220</v>
       </c>
-      <c r="O226" s="91" t="s">
+      <c r="O226" s="87" t="s">
         <v>1562</v>
       </c>
-      <c r="P226" s="91" t="s">
+      <c r="P226" s="87" t="s">
         <v>1562</v>
       </c>
-      <c r="Q226" s="92" t="s">
+      <c r="Q226" s="88" t="s">
         <v>1594</v>
       </c>
       <c r="R226" s="37" t="s">
@@ -42186,16 +42190,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[221][17]</v>
       </c>
-      <c r="N227" s="90">
+      <c r="N227" s="86">
         <v>221</v>
       </c>
-      <c r="O227" s="91" t="s">
+      <c r="O227" s="87" t="s">
         <v>1563</v>
       </c>
-      <c r="P227" s="91" t="s">
+      <c r="P227" s="87" t="s">
         <v>1563</v>
       </c>
-      <c r="Q227" s="92" t="s">
+      <c r="Q227" s="88" t="s">
         <v>1594</v>
       </c>
       <c r="R227" s="37" t="s">
@@ -42280,16 +42284,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[222][17]</v>
       </c>
-      <c r="N228" s="90">
+      <c r="N228" s="86">
         <v>222</v>
       </c>
-      <c r="O228" s="91" t="s">
+      <c r="O228" s="87" t="s">
         <v>1564</v>
       </c>
-      <c r="P228" s="91" t="s">
+      <c r="P228" s="87" t="s">
         <v>1564</v>
       </c>
-      <c r="Q228" s="92" t="s">
+      <c r="Q228" s="88" t="s">
         <v>1594</v>
       </c>
       <c r="R228" s="37" t="s">
@@ -42374,16 +42378,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[223][17]</v>
       </c>
-      <c r="N229" s="90">
+      <c r="N229" s="86">
         <v>223</v>
       </c>
-      <c r="O229" s="91" t="s">
+      <c r="O229" s="87" t="s">
         <v>1565</v>
       </c>
-      <c r="P229" s="91" t="s">
+      <c r="P229" s="87" t="s">
         <v>1565</v>
       </c>
-      <c r="Q229" s="92" t="s">
+      <c r="Q229" s="88" t="s">
         <v>1595</v>
       </c>
       <c r="R229" s="37" t="s">
@@ -42468,16 +42472,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[224][17]</v>
       </c>
-      <c r="N230" s="90">
+      <c r="N230" s="86">
         <v>224</v>
       </c>
-      <c r="O230" s="91" t="s">
+      <c r="O230" s="87" t="s">
         <v>1566</v>
       </c>
-      <c r="P230" s="91" t="s">
+      <c r="P230" s="87" t="s">
         <v>1566</v>
       </c>
-      <c r="Q230" s="92" t="s">
+      <c r="Q230" s="88" t="s">
         <v>1595</v>
       </c>
       <c r="R230" s="37" t="s">
@@ -42562,16 +42566,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[225][17]</v>
       </c>
-      <c r="N231" s="90">
+      <c r="N231" s="86">
         <v>225</v>
       </c>
-      <c r="O231" s="91" t="s">
+      <c r="O231" s="87" t="s">
         <v>1567</v>
       </c>
-      <c r="P231" s="91" t="s">
+      <c r="P231" s="87" t="s">
         <v>1567</v>
       </c>
-      <c r="Q231" s="92" t="s">
+      <c r="Q231" s="88" t="s">
         <v>1595</v>
       </c>
       <c r="R231" s="37" t="s">
@@ -42656,16 +42660,16 @@
         <f t="shared" ref="M232:M237" si="135">CONCATENATE("mp_ac[",N232,"][17]")</f>
         <v>mp_ac[226][17]</v>
       </c>
-      <c r="N232" s="90">
+      <c r="N232" s="86">
         <v>226</v>
       </c>
-      <c r="O232" s="91" t="s">
+      <c r="O232" s="87" t="s">
         <v>1568</v>
       </c>
-      <c r="P232" s="91" t="s">
+      <c r="P232" s="87" t="s">
         <v>1568</v>
       </c>
-      <c r="Q232" s="92" t="s">
+      <c r="Q232" s="88" t="s">
         <v>1596</v>
       </c>
       <c r="R232" s="37" t="s">
@@ -42750,16 +42754,16 @@
         <f t="shared" si="135"/>
         <v>mp_ac[227][17]</v>
       </c>
-      <c r="N233" s="90">
+      <c r="N233" s="86">
         <v>227</v>
       </c>
-      <c r="O233" s="91" t="s">
+      <c r="O233" s="87" t="s">
         <v>1569</v>
       </c>
-      <c r="P233" s="91" t="s">
+      <c r="P233" s="87" t="s">
         <v>1569</v>
       </c>
-      <c r="Q233" s="92" t="s">
+      <c r="Q233" s="88" t="s">
         <v>1596</v>
       </c>
       <c r="R233" s="37" t="s">
@@ -42844,16 +42848,16 @@
         <f t="shared" si="135"/>
         <v>mp_ac[228][17]</v>
       </c>
-      <c r="N234" s="90">
+      <c r="N234" s="86">
         <v>228</v>
       </c>
-      <c r="O234" s="91" t="s">
+      <c r="O234" s="87" t="s">
         <v>1570</v>
       </c>
-      <c r="P234" s="91" t="s">
+      <c r="P234" s="87" t="s">
         <v>1570</v>
       </c>
-      <c r="Q234" s="92" t="s">
+      <c r="Q234" s="88" t="s">
         <v>1596</v>
       </c>
       <c r="R234" s="37" t="s">
@@ -42938,16 +42942,16 @@
         <f t="shared" si="135"/>
         <v>mp_ac[229][17]</v>
       </c>
-      <c r="N235" s="90">
+      <c r="N235" s="86">
         <v>229</v>
       </c>
-      <c r="O235" s="91" t="s">
+      <c r="O235" s="87" t="s">
         <v>1571</v>
       </c>
-      <c r="P235" s="91" t="s">
+      <c r="P235" s="87" t="s">
         <v>1571</v>
       </c>
-      <c r="Q235" s="92" t="s">
+      <c r="Q235" s="88" t="s">
         <v>1597</v>
       </c>
       <c r="R235" s="37" t="s">
@@ -43032,16 +43036,16 @@
         <f t="shared" si="135"/>
         <v>mp_ac[230][17]</v>
       </c>
-      <c r="N236" s="90">
+      <c r="N236" s="86">
         <v>230</v>
       </c>
-      <c r="O236" s="91" t="s">
+      <c r="O236" s="87" t="s">
         <v>1572</v>
       </c>
-      <c r="P236" s="91" t="s">
+      <c r="P236" s="87" t="s">
         <v>1572</v>
       </c>
-      <c r="Q236" s="92" t="s">
+      <c r="Q236" s="88" t="s">
         <v>1597</v>
       </c>
       <c r="R236" s="37" t="s">
@@ -43126,16 +43130,16 @@
         <f t="shared" si="135"/>
         <v>mp_ac[231][17]</v>
       </c>
-      <c r="N237" s="90">
+      <c r="N237" s="86">
         <v>231</v>
       </c>
-      <c r="O237" s="91" t="s">
+      <c r="O237" s="87" t="s">
         <v>1573</v>
       </c>
-      <c r="P237" s="91" t="s">
+      <c r="P237" s="87" t="s">
         <v>1573</v>
       </c>
-      <c r="Q237" s="92" t="s">
+      <c r="Q237" s="88" t="s">
         <v>1597</v>
       </c>
       <c r="R237" s="37" t="s">
@@ -43220,16 +43224,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[232][17]</v>
       </c>
-      <c r="N238" s="90">
+      <c r="N238" s="86">
         <v>232</v>
       </c>
-      <c r="O238" s="91" t="s">
+      <c r="O238" s="87" t="s">
         <v>1574</v>
       </c>
-      <c r="P238" s="91" t="s">
+      <c r="P238" s="87" t="s">
         <v>1574</v>
       </c>
-      <c r="Q238" s="92" t="s">
+      <c r="Q238" s="88" t="s">
         <v>1598</v>
       </c>
       <c r="R238" s="37" t="s">
@@ -43314,16 +43318,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[233][17]</v>
       </c>
-      <c r="N239" s="90">
+      <c r="N239" s="86">
         <v>233</v>
       </c>
-      <c r="O239" s="91" t="s">
+      <c r="O239" s="87" t="s">
         <v>1575</v>
       </c>
-      <c r="P239" s="91" t="s">
+      <c r="P239" s="87" t="s">
         <v>1575</v>
       </c>
-      <c r="Q239" s="92" t="s">
+      <c r="Q239" s="88" t="s">
         <v>1598</v>
       </c>
       <c r="R239" s="37" t="s">
@@ -43408,16 +43412,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[234][17]</v>
       </c>
-      <c r="N240" s="90">
+      <c r="N240" s="86">
         <v>234</v>
       </c>
-      <c r="O240" s="91" t="s">
+      <c r="O240" s="87" t="s">
         <v>1576</v>
       </c>
-      <c r="P240" s="91" t="s">
+      <c r="P240" s="87" t="s">
         <v>1576</v>
       </c>
-      <c r="Q240" s="92" t="s">
+      <c r="Q240" s="88" t="s">
         <v>1598</v>
       </c>
       <c r="R240" s="37" t="s">
@@ -43502,16 +43506,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[235][17]</v>
       </c>
-      <c r="N241" s="90">
+      <c r="N241" s="86">
         <v>235</v>
       </c>
-      <c r="O241" s="91" t="s">
+      <c r="O241" s="87" t="s">
         <v>1577</v>
       </c>
-      <c r="P241" s="91" t="s">
+      <c r="P241" s="87" t="s">
         <v>1577</v>
       </c>
-      <c r="Q241" s="92" t="s">
+      <c r="Q241" s="88" t="s">
         <v>1599</v>
       </c>
       <c r="R241" s="37" t="s">
@@ -43596,16 +43600,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[236][17]</v>
       </c>
-      <c r="N242" s="90">
+      <c r="N242" s="86">
         <v>236</v>
       </c>
-      <c r="O242" s="91" t="s">
+      <c r="O242" s="87" t="s">
         <v>1578</v>
       </c>
-      <c r="P242" s="91" t="s">
+      <c r="P242" s="87" t="s">
         <v>1578</v>
       </c>
-      <c r="Q242" s="92" t="s">
+      <c r="Q242" s="88" t="s">
         <v>1599</v>
       </c>
       <c r="R242" s="37" t="s">
@@ -43690,16 +43694,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[237][17]</v>
       </c>
-      <c r="N243" s="90">
+      <c r="N243" s="86">
         <v>237</v>
       </c>
-      <c r="O243" s="91" t="s">
+      <c r="O243" s="87" t="s">
         <v>1579</v>
       </c>
-      <c r="P243" s="91" t="s">
+      <c r="P243" s="87" t="s">
         <v>1579</v>
       </c>
-      <c r="Q243" s="92" t="s">
+      <c r="Q243" s="88" t="s">
         <v>1599</v>
       </c>
       <c r="R243" s="37" t="s">
@@ -43784,16 +43788,16 @@
         <f t="shared" ref="M244:M249" si="143">CONCATENATE("mp_ac[",N244,"][17]")</f>
         <v>mp_ac[238][17]</v>
       </c>
-      <c r="N244" s="90">
+      <c r="N244" s="86">
         <v>238</v>
       </c>
-      <c r="O244" s="91" t="s">
+      <c r="O244" s="87" t="s">
         <v>1580</v>
       </c>
-      <c r="P244" s="91" t="s">
+      <c r="P244" s="87" t="s">
         <v>1580</v>
       </c>
-      <c r="Q244" s="92" t="s">
+      <c r="Q244" s="88" t="s">
         <v>1600</v>
       </c>
       <c r="R244" s="37" t="s">
@@ -43878,16 +43882,16 @@
         <f t="shared" si="143"/>
         <v>mp_ac[239][17]</v>
       </c>
-      <c r="N245" s="90">
+      <c r="N245" s="86">
         <v>239</v>
       </c>
-      <c r="O245" s="91" t="s">
+      <c r="O245" s="87" t="s">
         <v>1581</v>
       </c>
-      <c r="P245" s="91" t="s">
+      <c r="P245" s="87" t="s">
         <v>1581</v>
       </c>
-      <c r="Q245" s="92" t="s">
+      <c r="Q245" s="88" t="s">
         <v>1600</v>
       </c>
       <c r="R245" s="37" t="s">
@@ -43972,16 +43976,16 @@
         <f t="shared" si="143"/>
         <v>mp_ac[240][17]</v>
       </c>
-      <c r="N246" s="90">
+      <c r="N246" s="86">
         <v>240</v>
       </c>
-      <c r="O246" s="91" t="s">
+      <c r="O246" s="87" t="s">
         <v>1582</v>
       </c>
-      <c r="P246" s="91" t="s">
+      <c r="P246" s="87" t="s">
         <v>1582</v>
       </c>
-      <c r="Q246" s="92" t="s">
+      <c r="Q246" s="88" t="s">
         <v>1600</v>
       </c>
       <c r="R246" s="37" t="s">
@@ -44066,16 +44070,16 @@
         <f t="shared" si="143"/>
         <v>mp_ac[241][17]</v>
       </c>
-      <c r="N247" s="90">
+      <c r="N247" s="86">
         <v>241</v>
       </c>
-      <c r="O247" s="91" t="s">
+      <c r="O247" s="87" t="s">
         <v>1583</v>
       </c>
-      <c r="P247" s="91" t="s">
+      <c r="P247" s="87" t="s">
         <v>1583</v>
       </c>
-      <c r="Q247" s="92" t="s">
+      <c r="Q247" s="88" t="s">
         <v>1601</v>
       </c>
       <c r="R247" s="37" t="s">
@@ -44160,16 +44164,16 @@
         <f t="shared" si="143"/>
         <v>mp_ac[242][17]</v>
       </c>
-      <c r="N248" s="90">
+      <c r="N248" s="86">
         <v>242</v>
       </c>
-      <c r="O248" s="91" t="s">
+      <c r="O248" s="87" t="s">
         <v>1584</v>
       </c>
-      <c r="P248" s="91" t="s">
+      <c r="P248" s="87" t="s">
         <v>1584</v>
       </c>
-      <c r="Q248" s="92" t="s">
+      <c r="Q248" s="88" t="s">
         <v>1601</v>
       </c>
       <c r="R248" s="37" t="s">
@@ -44254,16 +44258,16 @@
         <f t="shared" si="143"/>
         <v>mp_ac[243][17]</v>
       </c>
-      <c r="N249" s="90">
+      <c r="N249" s="86">
         <v>243</v>
       </c>
-      <c r="O249" s="91" t="s">
+      <c r="O249" s="87" t="s">
         <v>1585</v>
       </c>
-      <c r="P249" s="91" t="s">
+      <c r="P249" s="87" t="s">
         <v>1585</v>
       </c>
-      <c r="Q249" s="92" t="s">
+      <c r="Q249" s="88" t="s">
         <v>1601</v>
       </c>
       <c r="R249" s="37" t="s">
@@ -44348,16 +44352,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[244][17]</v>
       </c>
-      <c r="N250" s="90">
+      <c r="N250" s="86">
         <v>244</v>
       </c>
-      <c r="O250" s="91" t="s">
+      <c r="O250" s="87" t="s">
         <v>1586</v>
       </c>
-      <c r="P250" s="91" t="s">
+      <c r="P250" s="87" t="s">
         <v>1586</v>
       </c>
-      <c r="Q250" s="92" t="s">
+      <c r="Q250" s="88" t="s">
         <v>1602</v>
       </c>
       <c r="R250" s="37" t="s">
@@ -44442,16 +44446,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[245][17]</v>
       </c>
-      <c r="N251" s="90">
+      <c r="N251" s="86">
         <v>245</v>
       </c>
-      <c r="O251" s="91" t="s">
+      <c r="O251" s="87" t="s">
         <v>1587</v>
       </c>
-      <c r="P251" s="91" t="s">
+      <c r="P251" s="87" t="s">
         <v>1587</v>
       </c>
-      <c r="Q251" s="92" t="s">
+      <c r="Q251" s="88" t="s">
         <v>1602</v>
       </c>
       <c r="R251" s="37" t="s">
@@ -44536,16 +44540,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[246][17]</v>
       </c>
-      <c r="N252" s="90">
+      <c r="N252" s="86">
         <v>246</v>
       </c>
-      <c r="O252" s="91" t="s">
+      <c r="O252" s="87" t="s">
         <v>1588</v>
       </c>
-      <c r="P252" s="91" t="s">
+      <c r="P252" s="87" t="s">
         <v>1588</v>
       </c>
-      <c r="Q252" s="92" t="s">
+      <c r="Q252" s="88" t="s">
         <v>1602</v>
       </c>
       <c r="R252" s="37" t="s">
@@ -44630,16 +44634,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[247][17]</v>
       </c>
-      <c r="N253" s="90">
+      <c r="N253" s="86">
         <v>247</v>
       </c>
-      <c r="O253" s="91" t="s">
+      <c r="O253" s="87" t="s">
         <v>1589</v>
       </c>
-      <c r="P253" s="91" t="s">
+      <c r="P253" s="87" t="s">
         <v>1589</v>
       </c>
-      <c r="Q253" s="92" t="s">
+      <c r="Q253" s="88" t="s">
         <v>1603</v>
       </c>
       <c r="R253" s="37" t="s">
@@ -44724,16 +44728,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[248][17]</v>
       </c>
-      <c r="N254" s="90">
+      <c r="N254" s="86">
         <v>248</v>
       </c>
-      <c r="O254" s="91" t="s">
+      <c r="O254" s="87" t="s">
         <v>1590</v>
       </c>
-      <c r="P254" s="91" t="s">
+      <c r="P254" s="87" t="s">
         <v>1590</v>
       </c>
-      <c r="Q254" s="92" t="s">
+      <c r="Q254" s="88" t="s">
         <v>1603</v>
       </c>
       <c r="R254" s="37" t="s">
@@ -44818,16 +44822,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[249][17]</v>
       </c>
-      <c r="N255" s="90">
+      <c r="N255" s="86">
         <v>249</v>
       </c>
-      <c r="O255" s="91" t="s">
+      <c r="O255" s="87" t="s">
         <v>1591</v>
       </c>
-      <c r="P255" s="91" t="s">
+      <c r="P255" s="87" t="s">
         <v>1591</v>
       </c>
-      <c r="Q255" s="92" t="s">
+      <c r="Q255" s="88" t="s">
         <v>1603</v>
       </c>
       <c r="R255" s="37" t="s">
@@ -44912,16 +44916,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[250][17]</v>
       </c>
-      <c r="N256" s="90">
+      <c r="N256" s="86">
         <v>250</v>
       </c>
-      <c r="O256" s="91" t="s">
+      <c r="O256" s="87" t="s">
         <v>1301</v>
       </c>
-      <c r="P256" s="91" t="s">
+      <c r="P256" s="87" t="s">
         <v>1301</v>
       </c>
-      <c r="Q256" s="92" t="s">
+      <c r="Q256" s="88" t="s">
         <v>1604</v>
       </c>
       <c r="R256" s="37" t="s">
@@ -45006,16 +45010,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[251][17]</v>
       </c>
-      <c r="N257" s="90">
+      <c r="N257" s="86">
         <v>251</v>
       </c>
-      <c r="O257" s="91" t="s">
+      <c r="O257" s="87" t="s">
         <v>1302</v>
       </c>
-      <c r="P257" s="91" t="s">
+      <c r="P257" s="87" t="s">
         <v>1302</v>
       </c>
-      <c r="Q257" s="92" t="s">
+      <c r="Q257" s="88" t="s">
         <v>1604</v>
       </c>
       <c r="R257" s="37" t="s">
@@ -45100,16 +45104,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[252][17]</v>
       </c>
-      <c r="N258" s="90">
+      <c r="N258" s="86">
         <v>252</v>
       </c>
-      <c r="O258" s="91" t="s">
+      <c r="O258" s="87" t="s">
         <v>1303</v>
       </c>
-      <c r="P258" s="91" t="s">
+      <c r="P258" s="87" t="s">
         <v>1303</v>
       </c>
-      <c r="Q258" s="92" t="s">
+      <c r="Q258" s="88" t="s">
         <v>1604</v>
       </c>
       <c r="R258" s="37" t="s">
@@ -45194,16 +45198,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[253][17]</v>
       </c>
-      <c r="N259" s="90">
+      <c r="N259" s="86">
         <v>253</v>
       </c>
-      <c r="O259" s="91" t="s">
+      <c r="O259" s="87" t="s">
         <v>1304</v>
       </c>
-      <c r="P259" s="91" t="s">
+      <c r="P259" s="87" t="s">
         <v>1304</v>
       </c>
-      <c r="Q259" s="92" t="s">
+      <c r="Q259" s="88" t="s">
         <v>1605</v>
       </c>
       <c r="R259" s="37" t="s">
@@ -45288,16 +45292,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[254][17]</v>
       </c>
-      <c r="N260" s="90">
+      <c r="N260" s="86">
         <v>254</v>
       </c>
-      <c r="O260" s="91" t="s">
+      <c r="O260" s="87" t="s">
         <v>1305</v>
       </c>
-      <c r="P260" s="91" t="s">
+      <c r="P260" s="87" t="s">
         <v>1305</v>
       </c>
-      <c r="Q260" s="92" t="s">
+      <c r="Q260" s="88" t="s">
         <v>1605</v>
       </c>
       <c r="R260" s="37" t="s">
@@ -45382,16 +45386,16 @@
         <f t="shared" si="119"/>
         <v>mp_ac[255][17]</v>
       </c>
-      <c r="N261" s="90">
+      <c r="N261" s="86">
         <v>255</v>
       </c>
-      <c r="O261" s="91" t="s">
+      <c r="O261" s="87" t="s">
         <v>1306</v>
       </c>
-      <c r="P261" s="91" t="s">
+      <c r="P261" s="87" t="s">
         <v>1306</v>
       </c>
-      <c r="Q261" s="92" t="s">
+      <c r="Q261" s="88" t="s">
         <v>1605</v>
       </c>
       <c r="R261" s="37" t="s">

</xml_diff>

<commit_message>
avanzando en la cotizacion tipo de un frente templado
</commit_message>
<xml_diff>
--- a/TRABAJOS-PYTHON/COTIZA_ALU_TEM/lista_materiales.xlsx
+++ b/TRABAJOS-PYTHON/COTIZA_ALU_TEM/lista_materiales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PcAsusZenbookRafita\Desktop\REPO_RAFAEL_ANTEQUERA\TRABAJOS-PYTHON\COTIZA_ALU_TEM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6965DC7E-4CB4-4E7C-9723-FEE60E43274E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{613BABF8-3F63-4605-80AB-CEFB34171A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1B3D5D76-0D2B-4247-8E51-F5AC57810600}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Costo M.P.yMat.'!$A$2:$F$94</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Costo M.P.yMat. (2)'!$A$2:$T$227</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Costo M.P.yMat. (2)'!$A$2:$T$231</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Costo M.P.yMat. (2)'!$2:$5</definedName>
   </definedNames>
   <calcPr calcId="191029" concurrentCalc="0"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3572" uniqueCount="1593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3596" uniqueCount="1603">
   <si>
     <t>ANALISIS DE COSTOS Y DETERMINACION DE PRECIOS DE VENTA (/i1,1/,84)</t>
   </si>
@@ -4737,66 +4737,6 @@
     <t xml:space="preserve">["PF10C", "PF10C", " PAÑOS FIJOS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
   </si>
   <si>
-    <t xml:space="preserve">["FTTS10", "CFTTS10", "FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["FTTS10C", "MOFTTS10C", "FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["FTCV10", "CFTCV10", "FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["FTCV10C", "MOFTCV10C", "FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["VC2H8", "CVC2H8", "VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["VC2H8C", "MOVC2H8C", "VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["VC4H8", "CVC4H8", "VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["VC4H8C", "MOVC4H8C", "VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["PVC2H10", "CPVC2H10", "PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["PVC2H10C", "MOPVC2H10C", "PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["PVC4H10", "CPVC4H10", "PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["PVC4H10C", "MOPVC4H10C", "PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["PB10", "CPB10", "PUERTAS BATIENTES CON O SIN FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["PB10C", "MOPB10C", "PUERTAS BATIENTES CON O SIN FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["OB", "OB", "OBRA  ", "obra"], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["CL", "CL", "CLIENTE  ", "cliente"], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["TE", "TE", "TELEFONO  ", "telefono"], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["DI", "DI", "DIRECCION  ", "direccion"], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["CO", "CO", "CORREO  ", "correo"], </t>
-  </si>
-  <si>
-    <t xml:space="preserve">["OBS", "OBS", "OBSERVACIONES  ", "observa"], </t>
-  </si>
-  <si>
     <t>PB10CF</t>
   </si>
   <si>
@@ -4819,6 +4759,96 @@
   </si>
   <si>
     <t xml:space="preserve">["PB10CFC", "PB10CFC", "PUERTAS BATIENTES CON FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 8 mm DE ESPESOR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 8 mm DE ESPESOR </t>
+  </si>
+  <si>
+    <t>FTCV8</t>
+  </si>
+  <si>
+    <t>FTCV8C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["OB", "OB", "OBRA  ", "obra",  ,  ,  ,  ,  ,  , " ",  ,  ,  ,  ,  ,  ,  ,  ], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["CL", "CL", "CLIENTE  ", "cliente",  ,  ,  ,  ,  ,  , " ",  ,  ,  ,  ,  ,  ,  ,  ], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["TE", "TE", "TELEFONO  ", "telefono",  ,  ,  ,  ,  ,  , " ",  ,  ,  ,  ,  ,  ,  ,  ], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["DI", "DI", "DIRECCION  ", "direccion",  ,  ,  ,  ,  ,  , " ",  ,  ,  ,  ,  ,  ,  ,  ], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["CO", "CO", "CORREO  ", "correo",  ,  ,  ,  ,  ,  , " ",  ,  ,  ,  ,  ,  ,  ,  ], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["OBS", "OBS", "OBSERVACIONES  ", "observa",  ,  ,  ,  ,  ,  , " ",  ,  ,  ,  ,  ,  ,  ,  ], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["FTCV8", "FTCV8", "FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["FTCV8C", "FTCV8C", "FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["FTTS10", "FTTS10", "FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["FTTS10C", "FTTS10C", "FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["FTCV8", "FTCV8", "FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["FTCV8C", "FTCV8C", "FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["FTCV10", "FTCV10", "FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["FTCV10C", "FTCV10C", "FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["VC2H8", "VC2H8", "VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["VC2H8C", "VC2H8C", "VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["VC4H8", "VC4H8", "VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["VC4H8C", "VC4H8C", "VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["PVC2H10", "PVC2H10", "PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["PVC2H10C", "PVC2H10C", "PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["PVC4H10", "PVC4H10", "PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["PVC4H10C", "PVC4H10C", "PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["PB10", "PB10", "PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t xml:space="preserve">["PB10C", "PB10C", "PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
   </si>
 </sst>
 </file>
@@ -5310,12 +5340,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -5357,6 +5381,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -5984,10 +6014,10 @@
       <c r="D3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="80" t="s">
+      <c r="E3" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="80"/>
+      <c r="F3" s="94"/>
       <c r="G3" s="48" t="s">
         <v>496</v>
       </c>
@@ -14515,13 +14545,13 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB227"/>
+  <dimension ref="A1:AB231"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="27.6" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="72" customWidth="1"/>
     <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" customWidth="1"/>
-    <col min="4" max="4" width="75.5546875" style="95" customWidth="1"/>
+    <col min="4" max="4" width="75.5546875" style="93" customWidth="1"/>
     <col min="5" max="5" width="10.77734375" style="28" customWidth="1"/>
     <col min="6" max="7" width="11.5546875" style="20" bestFit="1" customWidth="1"/>
     <col min="8" max="11" width="11.77734375" style="27" bestFit="1" customWidth="1"/>
@@ -14537,7 +14567,7 @@
   <sheetData>
     <row r="1" spans="1:28" s="1" customFormat="1" ht="37.200000000000003" x14ac:dyDescent="0.45">
       <c r="A1" s="71"/>
-      <c r="D1" s="82" t="s">
+      <c r="D1" s="80" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="3"/>
@@ -14562,7 +14592,7 @@
       <c r="C2" s="73">
         <v>1</v>
       </c>
-      <c r="D2" s="83">
+      <c r="D2" s="81">
         <v>2</v>
       </c>
       <c r="E2" s="73">
@@ -14617,23 +14647,23 @@
       <c r="V2" s="75"/>
     </row>
     <row r="3" spans="1:28" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="81"/>
+      <c r="A3" s="95"/>
       <c r="B3" s="47" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="84" t="s">
+      <c r="D3" s="82" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="80" t="s">
+      <c r="F3" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="80"/>
+      <c r="G3" s="94"/>
       <c r="H3" s="48" t="s">
         <v>496</v>
       </c>
@@ -14677,12 +14707,12 @@
       <c r="V3" s="6"/>
     </row>
     <row r="4" spans="1:28" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="81"/>
+      <c r="A4" s="95"/>
       <c r="B4" s="49"/>
       <c r="C4" s="49" t="s">
         <v>320</v>
       </c>
-      <c r="D4" s="85"/>
+      <c r="D4" s="83"/>
       <c r="E4" s="50"/>
       <c r="F4" s="49" t="s">
         <v>6</v>
@@ -14715,10 +14745,10 @@
       <c r="V4" s="6"/>
     </row>
     <row r="5" spans="1:28" s="1" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="81"/>
+      <c r="A5" s="95"/>
       <c r="B5" s="51"/>
       <c r="C5" s="51"/>
-      <c r="D5" s="86"/>
+      <c r="D5" s="84"/>
       <c r="E5" s="52"/>
       <c r="F5" s="51" t="s">
         <v>7</v>
@@ -14760,7 +14790,7 @@
       <c r="C6" s="25" t="s">
         <v>1280</v>
       </c>
-      <c r="D6" s="87" t="s">
+      <c r="D6" s="85" t="s">
         <v>1281</v>
       </c>
       <c r="E6" s="25" t="s">
@@ -14832,7 +14862,7 @@
       <c r="C7" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="88" t="s">
+      <c r="D7" s="86" t="s">
         <v>322</v>
       </c>
       <c r="E7" s="35" t="s">
@@ -14909,7 +14939,7 @@
       <c r="C8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="88" t="s">
+      <c r="D8" s="86" t="s">
         <v>323</v>
       </c>
       <c r="E8" s="35" t="s">
@@ -14986,7 +15016,7 @@
       <c r="C9" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="89" t="s">
+      <c r="D9" s="87" t="s">
         <v>1321</v>
       </c>
       <c r="E9" s="37" t="s">
@@ -15063,7 +15093,7 @@
       <c r="C10" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="88" t="s">
+      <c r="D10" s="86" t="s">
         <v>1357</v>
       </c>
       <c r="E10" s="35" t="s">
@@ -15140,7 +15170,7 @@
       <c r="C11" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="88" t="s">
+      <c r="D11" s="86" t="s">
         <v>1358</v>
       </c>
       <c r="E11" s="35" t="s">
@@ -15217,7 +15247,7 @@
       <c r="C12" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="89" t="s">
+      <c r="D12" s="87" t="s">
         <v>327</v>
       </c>
       <c r="E12" s="37" t="s">
@@ -15294,7 +15324,7 @@
       <c r="C13" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="89" t="s">
+      <c r="D13" s="87" t="s">
         <v>328</v>
       </c>
       <c r="E13" s="37" t="s">
@@ -15371,7 +15401,7 @@
       <c r="C14" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="88" t="s">
+      <c r="D14" s="86" t="s">
         <v>329</v>
       </c>
       <c r="E14" s="35" t="s">
@@ -15448,7 +15478,7 @@
       <c r="C15" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="88" t="s">
+      <c r="D15" s="86" t="s">
         <v>330</v>
       </c>
       <c r="E15" s="35" t="s">
@@ -15525,7 +15555,7 @@
       <c r="C16" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="88" t="s">
+      <c r="D16" s="86" t="s">
         <v>331</v>
       </c>
       <c r="E16" s="35" t="s">
@@ -15602,7 +15632,7 @@
       <c r="C17" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D17" s="89" t="s">
+      <c r="D17" s="87" t="s">
         <v>332</v>
       </c>
       <c r="E17" s="37" t="s">
@@ -15679,7 +15709,7 @@
       <c r="C18" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="89" t="s">
+      <c r="D18" s="87" t="s">
         <v>333</v>
       </c>
       <c r="E18" s="37" t="s">
@@ -15756,7 +15786,7 @@
       <c r="C19" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="89" t="s">
+      <c r="D19" s="87" t="s">
         <v>334</v>
       </c>
       <c r="E19" s="37" t="s">
@@ -15833,7 +15863,7 @@
       <c r="C20" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="89" t="s">
+      <c r="D20" s="87" t="s">
         <v>335</v>
       </c>
       <c r="E20" s="37" t="s">
@@ -15910,7 +15940,7 @@
       <c r="C21" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="89" t="s">
+      <c r="D21" s="87" t="s">
         <v>336</v>
       </c>
       <c r="E21" s="37" t="s">
@@ -15987,7 +16017,7 @@
       <c r="C22" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D22" s="89" t="s">
+      <c r="D22" s="87" t="s">
         <v>1322</v>
       </c>
       <c r="E22" s="37" t="s">
@@ -16064,7 +16094,7 @@
       <c r="C23" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D23" s="88" t="s">
+      <c r="D23" s="86" t="s">
         <v>338</v>
       </c>
       <c r="E23" s="35" t="s">
@@ -16141,7 +16171,7 @@
       <c r="C24" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="88" t="s">
+      <c r="D24" s="86" t="s">
         <v>339</v>
       </c>
       <c r="E24" s="35" t="s">
@@ -16218,7 +16248,7 @@
       <c r="C25" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="D25" s="89" t="s">
+      <c r="D25" s="87" t="s">
         <v>340</v>
       </c>
       <c r="E25" s="37" t="s">
@@ -16295,7 +16325,7 @@
       <c r="C26" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D26" s="89" t="s">
+      <c r="D26" s="87" t="s">
         <v>341</v>
       </c>
       <c r="E26" s="37" t="s">
@@ -16372,7 +16402,7 @@
       <c r="C27" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D27" s="89" t="s">
+      <c r="D27" s="87" t="s">
         <v>342</v>
       </c>
       <c r="E27" s="37" t="s">
@@ -16449,7 +16479,7 @@
       <c r="C28" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="88" t="s">
+      <c r="D28" s="86" t="s">
         <v>343</v>
       </c>
       <c r="E28" s="35" t="s">
@@ -16526,7 +16556,7 @@
       <c r="C29" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D29" s="88" t="s">
+      <c r="D29" s="86" t="s">
         <v>344</v>
       </c>
       <c r="E29" s="35" t="s">
@@ -16603,7 +16633,7 @@
       <c r="C30" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="89" t="s">
+      <c r="D30" s="87" t="s">
         <v>345</v>
       </c>
       <c r="E30" s="37" t="s">
@@ -16680,7 +16710,7 @@
       <c r="C31" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D31" s="89" t="s">
+      <c r="D31" s="87" t="s">
         <v>346</v>
       </c>
       <c r="E31" s="37" t="s">
@@ -16757,7 +16787,7 @@
       <c r="C32" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="89" t="s">
+      <c r="D32" s="87" t="s">
         <v>347</v>
       </c>
       <c r="E32" s="37" t="s">
@@ -16834,7 +16864,7 @@
       <c r="C33" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="D33" s="89" t="s">
+      <c r="D33" s="87" t="s">
         <v>348</v>
       </c>
       <c r="E33" s="37" t="s">
@@ -16911,7 +16941,7 @@
       <c r="C34" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D34" s="89" t="s">
+      <c r="D34" s="87" t="s">
         <v>349</v>
       </c>
       <c r="E34" s="37" t="s">
@@ -16988,7 +17018,7 @@
       <c r="C35" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D35" s="88" t="s">
+      <c r="D35" s="86" t="s">
         <v>350</v>
       </c>
       <c r="E35" s="35" t="s">
@@ -17065,7 +17095,7 @@
       <c r="C36" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D36" s="88" t="s">
+      <c r="D36" s="86" t="s">
         <v>351</v>
       </c>
       <c r="E36" s="35" t="s">
@@ -17142,7 +17172,7 @@
       <c r="C37" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D37" s="88" t="s">
+      <c r="D37" s="86" t="s">
         <v>352</v>
       </c>
       <c r="E37" s="35" t="s">
@@ -17219,7 +17249,7 @@
       <c r="C38" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D38" s="89" t="s">
+      <c r="D38" s="87" t="s">
         <v>353</v>
       </c>
       <c r="E38" s="37" t="s">
@@ -17296,7 +17326,7 @@
       <c r="C39" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="D39" s="89" t="s">
+      <c r="D39" s="87" t="s">
         <v>354</v>
       </c>
       <c r="E39" s="37" t="s">
@@ -17373,7 +17403,7 @@
       <c r="C40" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="D40" s="89" t="s">
+      <c r="D40" s="87" t="s">
         <v>355</v>
       </c>
       <c r="E40" s="37" t="s">
@@ -17450,7 +17480,7 @@
       <c r="C41" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D41" s="89" t="s">
+      <c r="D41" s="87" t="s">
         <v>356</v>
       </c>
       <c r="E41" s="37" t="s">
@@ -17527,7 +17557,7 @@
       <c r="C42" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D42" s="89" t="s">
+      <c r="D42" s="87" t="s">
         <v>357</v>
       </c>
       <c r="E42" s="37" t="s">
@@ -17604,7 +17634,7 @@
       <c r="C43" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="D43" s="89" t="s">
+      <c r="D43" s="87" t="s">
         <v>358</v>
       </c>
       <c r="E43" s="37" t="s">
@@ -17681,7 +17711,7 @@
       <c r="C44" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D44" s="89" t="s">
+      <c r="D44" s="87" t="s">
         <v>359</v>
       </c>
       <c r="E44" s="37" t="s">
@@ -17758,7 +17788,7 @@
       <c r="C45" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="D45" s="88" t="s">
+      <c r="D45" s="86" t="s">
         <v>360</v>
       </c>
       <c r="E45" s="35" t="s">
@@ -17835,7 +17865,7 @@
       <c r="C46" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="D46" s="88" t="s">
+      <c r="D46" s="86" t="s">
         <v>361</v>
       </c>
       <c r="E46" s="35" t="s">
@@ -17912,7 +17942,7 @@
       <c r="C47" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D47" s="88" t="s">
+      <c r="D47" s="86" t="s">
         <v>362</v>
       </c>
       <c r="E47" s="35" t="s">
@@ -17989,7 +18019,7 @@
       <c r="C48" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="D48" s="88" t="s">
+      <c r="D48" s="86" t="s">
         <v>363</v>
       </c>
       <c r="E48" s="35" t="s">
@@ -18066,7 +18096,7 @@
       <c r="C49" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="D49" s="88" t="s">
+      <c r="D49" s="86" t="s">
         <v>364</v>
       </c>
       <c r="E49" s="35" t="s">
@@ -18143,7 +18173,7 @@
       <c r="C50" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="D50" s="88" t="s">
+      <c r="D50" s="86" t="s">
         <v>365</v>
       </c>
       <c r="E50" s="35" t="s">
@@ -18220,7 +18250,7 @@
       <c r="C51" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="D51" s="88" t="s">
+      <c r="D51" s="86" t="s">
         <v>366</v>
       </c>
       <c r="E51" s="35" t="s">
@@ -18297,7 +18327,7 @@
       <c r="C52" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="D52" s="88" t="s">
+      <c r="D52" s="86" t="s">
         <v>367</v>
       </c>
       <c r="E52" s="35" t="s">
@@ -18374,7 +18404,7 @@
       <c r="C53" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="D53" s="88" t="s">
+      <c r="D53" s="86" t="s">
         <v>368</v>
       </c>
       <c r="E53" s="35" t="s">
@@ -18451,7 +18481,7 @@
       <c r="C54" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D54" s="88" t="s">
+      <c r="D54" s="86" t="s">
         <v>369</v>
       </c>
       <c r="E54" s="35" t="s">
@@ -18528,7 +18558,7 @@
       <c r="C55" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D55" s="88" t="s">
+      <c r="D55" s="86" t="s">
         <v>370</v>
       </c>
       <c r="E55" s="35" t="s">
@@ -18605,7 +18635,7 @@
       <c r="C56" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D56" s="88" t="s">
+      <c r="D56" s="86" t="s">
         <v>371</v>
       </c>
       <c r="E56" s="35" t="s">
@@ -18682,7 +18712,7 @@
       <c r="C57" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="D57" s="88" t="s">
+      <c r="D57" s="86" t="s">
         <v>372</v>
       </c>
       <c r="E57" s="35" t="s">
@@ -18759,7 +18789,7 @@
       <c r="C58" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="D58" s="88" t="s">
+      <c r="D58" s="86" t="s">
         <v>373</v>
       </c>
       <c r="E58" s="35" t="s">
@@ -18836,7 +18866,7 @@
       <c r="C59" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D59" s="88" t="s">
+      <c r="D59" s="86" t="s">
         <v>374</v>
       </c>
       <c r="E59" s="35" t="s">
@@ -18913,7 +18943,7 @@
       <c r="C60" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D60" s="88" t="s">
+      <c r="D60" s="86" t="s">
         <v>375</v>
       </c>
       <c r="E60" s="35" t="s">
@@ -18990,7 +19020,7 @@
       <c r="C61" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="D61" s="88" t="s">
+      <c r="D61" s="86" t="s">
         <v>376</v>
       </c>
       <c r="E61" s="35" t="s">
@@ -19067,7 +19097,7 @@
       <c r="C62" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="D62" s="88" t="s">
+      <c r="D62" s="86" t="s">
         <v>377</v>
       </c>
       <c r="E62" s="35" t="s">
@@ -19144,7 +19174,7 @@
       <c r="C63" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="D63" s="88" t="s">
+      <c r="D63" s="86" t="s">
         <v>378</v>
       </c>
       <c r="E63" s="35" t="s">
@@ -19221,7 +19251,7 @@
       <c r="C64" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D64" s="88" t="s">
+      <c r="D64" s="86" t="s">
         <v>379</v>
       </c>
       <c r="E64" s="35" t="s">
@@ -19298,7 +19328,7 @@
       <c r="C65" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="D65" s="88" t="s">
+      <c r="D65" s="86" t="s">
         <v>380</v>
       </c>
       <c r="E65" s="35" t="s">
@@ -19375,7 +19405,7 @@
       <c r="C66" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D66" s="88" t="s">
+      <c r="D66" s="86" t="s">
         <v>381</v>
       </c>
       <c r="E66" s="35" t="s">
@@ -19452,7 +19482,7 @@
       <c r="C67" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D67" s="88" t="s">
+      <c r="D67" s="86" t="s">
         <v>382</v>
       </c>
       <c r="E67" s="35" t="s">
@@ -19529,7 +19559,7 @@
       <c r="C68" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="D68" s="88" t="s">
+      <c r="D68" s="86" t="s">
         <v>383</v>
       </c>
       <c r="E68" s="35" t="s">
@@ -19606,7 +19636,7 @@
       <c r="C69" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="D69" s="88" t="s">
+      <c r="D69" s="86" t="s">
         <v>384</v>
       </c>
       <c r="E69" s="35" t="s">
@@ -19683,7 +19713,7 @@
       <c r="C70" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D70" s="88" t="s">
+      <c r="D70" s="86" t="s">
         <v>385</v>
       </c>
       <c r="E70" s="35" t="s">
@@ -19760,7 +19790,7 @@
       <c r="C71" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="D71" s="88" t="s">
+      <c r="D71" s="86" t="s">
         <v>386</v>
       </c>
       <c r="E71" s="35" t="s">
@@ -19837,7 +19867,7 @@
       <c r="C72" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="D72" s="88" t="s">
+      <c r="D72" s="86" t="s">
         <v>387</v>
       </c>
       <c r="E72" s="35" t="s">
@@ -19914,7 +19944,7 @@
       <c r="C73" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D73" s="88" t="s">
+      <c r="D73" s="86" t="s">
         <v>388</v>
       </c>
       <c r="E73" s="35" t="s">
@@ -19991,7 +20021,7 @@
       <c r="C74" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="D74" s="88" t="s">
+      <c r="D74" s="86" t="s">
         <v>389</v>
       </c>
       <c r="E74" s="35" t="s">
@@ -20068,7 +20098,7 @@
       <c r="C75" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="D75" s="88" t="s">
+      <c r="D75" s="86" t="s">
         <v>390</v>
       </c>
       <c r="E75" s="35" t="s">
@@ -20145,7 +20175,7 @@
       <c r="C76" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="D76" s="88" t="s">
+      <c r="D76" s="86" t="s">
         <v>391</v>
       </c>
       <c r="E76" s="35" t="s">
@@ -20222,7 +20252,7 @@
       <c r="C77" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="D77" s="88" t="s">
+      <c r="D77" s="86" t="s">
         <v>392</v>
       </c>
       <c r="E77" s="35" t="s">
@@ -20299,7 +20329,7 @@
       <c r="C78" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D78" s="88" t="s">
+      <c r="D78" s="86" t="s">
         <v>393</v>
       </c>
       <c r="E78" s="35" t="s">
@@ -20376,7 +20406,7 @@
       <c r="C79" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="D79" s="88" t="s">
+      <c r="D79" s="86" t="s">
         <v>394</v>
       </c>
       <c r="E79" s="35" t="s">
@@ -20453,7 +20483,7 @@
       <c r="C80" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="D80" s="88" t="s">
+      <c r="D80" s="86" t="s">
         <v>395</v>
       </c>
       <c r="E80" s="35" t="s">
@@ -20530,7 +20560,7 @@
       <c r="C81" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D81" s="88" t="s">
+      <c r="D81" s="86" t="s">
         <v>396</v>
       </c>
       <c r="E81" s="35" t="s">
@@ -20607,7 +20637,7 @@
       <c r="C82" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="D82" s="89" t="s">
+      <c r="D82" s="87" t="s">
         <v>397</v>
       </c>
       <c r="E82" s="37" t="s">
@@ -20684,7 +20714,7 @@
       <c r="C83" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D83" s="89" t="s">
+      <c r="D83" s="87" t="s">
         <v>398</v>
       </c>
       <c r="E83" s="37" t="s">
@@ -20761,7 +20791,7 @@
       <c r="C84" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="D84" s="88" t="s">
+      <c r="D84" s="86" t="s">
         <v>1305</v>
       </c>
       <c r="E84" s="37" t="s">
@@ -20838,7 +20868,7 @@
       <c r="C85" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="D85" s="89" t="s">
+      <c r="D85" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E85" s="37" t="s">
@@ -20915,7 +20945,7 @@
       <c r="C86" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="D86" s="89" t="s">
+      <c r="D86" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E86" s="37" t="s">
@@ -20992,7 +21022,7 @@
       <c r="C87" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="D87" s="89" t="s">
+      <c r="D87" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E87" s="37" t="s">
@@ -21069,7 +21099,7 @@
       <c r="C88" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="D88" s="89" t="s">
+      <c r="D88" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E88" s="37" t="s">
@@ -21146,7 +21176,7 @@
       <c r="C89" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="D89" s="89" t="s">
+      <c r="D89" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E89" s="37" t="s">
@@ -21223,7 +21253,7 @@
       <c r="C90" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D90" s="89" t="s">
+      <c r="D90" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E90" s="37" t="s">
@@ -21300,7 +21330,7 @@
       <c r="C91" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="D91" s="89" t="s">
+      <c r="D91" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E91" s="37" t="s">
@@ -21377,7 +21407,7 @@
       <c r="C92" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="D92" s="89" t="s">
+      <c r="D92" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E92" s="37" t="s">
@@ -21454,7 +21484,7 @@
       <c r="C93" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="D93" s="89" t="s">
+      <c r="D93" s="87" t="s">
         <v>1304</v>
       </c>
       <c r="E93" s="37" t="s">
@@ -21531,7 +21561,7 @@
       <c r="C94" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="D94" s="89" t="s">
+      <c r="D94" s="87" t="s">
         <v>399</v>
       </c>
       <c r="E94" s="37" t="s">
@@ -21608,7 +21638,7 @@
       <c r="C95" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="D95" s="89" t="s">
+      <c r="D95" s="87" t="s">
         <v>400</v>
       </c>
       <c r="E95" s="37" t="s">
@@ -21685,7 +21715,7 @@
       <c r="C96" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D96" s="89" t="s">
+      <c r="D96" s="87" t="s">
         <v>401</v>
       </c>
       <c r="E96" s="37" t="s">
@@ -21762,7 +21792,7 @@
       <c r="C97" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="D97" s="89" t="s">
+      <c r="D97" s="87" t="s">
         <v>402</v>
       </c>
       <c r="E97" s="37" t="s">
@@ -21839,7 +21869,7 @@
       <c r="C98" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="D98" s="89" t="s">
+      <c r="D98" s="87" t="s">
         <v>403</v>
       </c>
       <c r="E98" s="37" t="s">
@@ -21916,7 +21946,7 @@
       <c r="C99" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="D99" s="89" t="s">
+      <c r="D99" s="87" t="s">
         <v>404</v>
       </c>
       <c r="E99" s="37" t="s">
@@ -21993,7 +22023,7 @@
       <c r="C100" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D100" s="89" t="s">
+      <c r="D100" s="87" t="s">
         <v>405</v>
       </c>
       <c r="E100" s="37" t="s">
@@ -22070,7 +22100,7 @@
       <c r="C101" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="D101" s="89" t="s">
+      <c r="D101" s="87" t="s">
         <v>406</v>
       </c>
       <c r="E101" s="37" t="s">
@@ -22147,7 +22177,7 @@
       <c r="C102" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="D102" s="89" t="s">
+      <c r="D102" s="87" t="s">
         <v>407</v>
       </c>
       <c r="E102" s="37" t="s">
@@ -22224,7 +22254,7 @@
       <c r="C103" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="D103" s="89" t="s">
+      <c r="D103" s="87" t="s">
         <v>408</v>
       </c>
       <c r="E103" s="37" t="s">
@@ -22301,7 +22331,7 @@
       <c r="C104" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="D104" s="89" t="s">
+      <c r="D104" s="87" t="s">
         <v>409</v>
       </c>
       <c r="E104" s="37" t="s">
@@ -22378,7 +22408,7 @@
       <c r="C105" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="D105" s="89" t="s">
+      <c r="D105" s="87" t="s">
         <v>410</v>
       </c>
       <c r="E105" s="37" t="s">
@@ -22455,7 +22485,7 @@
       <c r="C106" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="D106" s="89" t="s">
+      <c r="D106" s="87" t="s">
         <v>411</v>
       </c>
       <c r="E106" s="37" t="s">
@@ -22532,7 +22562,7 @@
       <c r="C107" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="D107" s="89" t="s">
+      <c r="D107" s="87" t="s">
         <v>412</v>
       </c>
       <c r="E107" s="37" t="s">
@@ -22609,7 +22639,7 @@
       <c r="C108" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="D108" s="89" t="s">
+      <c r="D108" s="87" t="s">
         <v>413</v>
       </c>
       <c r="E108" s="37" t="s">
@@ -22686,7 +22716,7 @@
       <c r="C109" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D109" s="89" t="s">
+      <c r="D109" s="87" t="s">
         <v>414</v>
       </c>
       <c r="E109" s="37" t="s">
@@ -22763,7 +22793,7 @@
       <c r="C110" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="D110" s="89" t="s">
+      <c r="D110" s="87" t="s">
         <v>415</v>
       </c>
       <c r="E110" s="37" t="s">
@@ -22840,7 +22870,7 @@
       <c r="C111" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="D111" s="89" t="s">
+      <c r="D111" s="87" t="s">
         <v>416</v>
       </c>
       <c r="E111" s="37" t="s">
@@ -22917,7 +22947,7 @@
       <c r="C112" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="D112" s="89" t="s">
+      <c r="D112" s="87" t="s">
         <v>1323</v>
       </c>
       <c r="E112" s="37" t="s">
@@ -22994,7 +23024,7 @@
       <c r="C113" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="D113" s="89" t="s">
+      <c r="D113" s="87" t="s">
         <v>1324</v>
       </c>
       <c r="E113" s="37" t="s">
@@ -23071,7 +23101,7 @@
       <c r="C114" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="D114" s="89" t="s">
+      <c r="D114" s="87" t="s">
         <v>1325</v>
       </c>
       <c r="E114" s="37" t="s">
@@ -23148,7 +23178,7 @@
       <c r="C115" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="D115" s="89" t="s">
+      <c r="D115" s="87" t="s">
         <v>332</v>
       </c>
       <c r="E115" s="37" t="s">
@@ -23225,7 +23255,7 @@
       <c r="C116" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="D116" s="89" t="s">
+      <c r="D116" s="87" t="s">
         <v>420</v>
       </c>
       <c r="E116" s="37" t="s">
@@ -23302,7 +23332,7 @@
       <c r="C117" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="D117" s="89" t="s">
+      <c r="D117" s="87" t="s">
         <v>421</v>
       </c>
       <c r="E117" s="37" t="s">
@@ -23379,7 +23409,7 @@
       <c r="C118" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="D118" s="89" t="s">
+      <c r="D118" s="87" t="s">
         <v>422</v>
       </c>
       <c r="E118" s="37" t="s">
@@ -23456,7 +23486,7 @@
       <c r="C119" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D119" s="89" t="s">
+      <c r="D119" s="87" t="s">
         <v>423</v>
       </c>
       <c r="E119" s="37" t="s">
@@ -23533,7 +23563,7 @@
       <c r="C120" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="D120" s="89" t="s">
+      <c r="D120" s="87" t="s">
         <v>424</v>
       </c>
       <c r="E120" s="37" t="s">
@@ -23610,7 +23640,7 @@
       <c r="C121" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="D121" s="89" t="s">
+      <c r="D121" s="87" t="s">
         <v>425</v>
       </c>
       <c r="E121" s="37" t="s">
@@ -23687,7 +23717,7 @@
       <c r="C122" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="D122" s="89" t="s">
+      <c r="D122" s="87" t="s">
         <v>426</v>
       </c>
       <c r="E122" s="37" t="s">
@@ -23764,7 +23794,7 @@
       <c r="C123" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="D123" s="89" t="s">
+      <c r="D123" s="87" t="s">
         <v>427</v>
       </c>
       <c r="E123" s="37" t="s">
@@ -23841,7 +23871,7 @@
       <c r="C124" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="D124" s="89" t="s">
+      <c r="D124" s="87" t="s">
         <v>428</v>
       </c>
       <c r="E124" s="37" t="s">
@@ -23918,7 +23948,7 @@
       <c r="C125" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="D125" s="89" t="s">
+      <c r="D125" s="87" t="s">
         <v>429</v>
       </c>
       <c r="E125" s="37" t="s">
@@ -23995,7 +24025,7 @@
       <c r="C126" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D126" s="89" t="s">
+      <c r="D126" s="87" t="s">
         <v>430</v>
       </c>
       <c r="E126" s="37" t="s">
@@ -24072,7 +24102,7 @@
       <c r="C127" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="D127" s="89" t="s">
+      <c r="D127" s="87" t="s">
         <v>431</v>
       </c>
       <c r="E127" s="37" t="s">
@@ -24149,7 +24179,7 @@
       <c r="C128" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="D128" s="89" t="s">
+      <c r="D128" s="87" t="s">
         <v>432</v>
       </c>
       <c r="E128" s="37" t="s">
@@ -24226,7 +24256,7 @@
       <c r="C129" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="D129" s="89" t="s">
+      <c r="D129" s="87" t="s">
         <v>433</v>
       </c>
       <c r="E129" s="37" t="s">
@@ -24303,7 +24333,7 @@
       <c r="C130" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="D130" s="89" t="s">
+      <c r="D130" s="87" t="s">
         <v>434</v>
       </c>
       <c r="E130" s="37" t="s">
@@ -24380,7 +24410,7 @@
       <c r="C131" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="D131" s="89" t="s">
+      <c r="D131" s="87" t="s">
         <v>435</v>
       </c>
       <c r="E131" s="37" t="s">
@@ -24457,7 +24487,7 @@
       <c r="C132" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="D132" s="89" t="s">
+      <c r="D132" s="87" t="s">
         <v>436</v>
       </c>
       <c r="E132" s="37" t="s">
@@ -24534,7 +24564,7 @@
       <c r="C133" s="11" t="s">
         <v>144</v>
       </c>
-      <c r="D133" s="89" t="s">
+      <c r="D133" s="87" t="s">
         <v>437</v>
       </c>
       <c r="E133" s="37" t="s">
@@ -24611,7 +24641,7 @@
       <c r="C134" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="D134" s="89" t="s">
+      <c r="D134" s="87" t="s">
         <v>438</v>
       </c>
       <c r="E134" s="37" t="s">
@@ -24688,7 +24718,7 @@
       <c r="C135" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="D135" s="89" t="s">
+      <c r="D135" s="87" t="s">
         <v>439</v>
       </c>
       <c r="E135" s="37" t="s">
@@ -24765,7 +24795,7 @@
       <c r="C136" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="D136" s="89" t="s">
+      <c r="D136" s="87" t="s">
         <v>440</v>
       </c>
       <c r="E136" s="37" t="s">
@@ -24842,7 +24872,7 @@
       <c r="C137" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="D137" s="89" t="s">
+      <c r="D137" s="87" t="s">
         <v>441</v>
       </c>
       <c r="E137" s="37" t="s">
@@ -24919,7 +24949,7 @@
       <c r="C138" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="D138" s="89" t="s">
+      <c r="D138" s="87" t="s">
         <v>442</v>
       </c>
       <c r="E138" s="37" t="s">
@@ -24996,7 +25026,7 @@
       <c r="C139" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="D139" s="89" t="s">
+      <c r="D139" s="87" t="s">
         <v>443</v>
       </c>
       <c r="E139" s="37" t="s">
@@ -25073,7 +25103,7 @@
       <c r="C140" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="D140" s="89" t="s">
+      <c r="D140" s="87" t="s">
         <v>444</v>
       </c>
       <c r="E140" s="37" t="s">
@@ -25150,7 +25180,7 @@
       <c r="C141" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="D141" s="89" t="s">
+      <c r="D141" s="87" t="s">
         <v>445</v>
       </c>
       <c r="E141" s="37" t="s">
@@ -25227,7 +25257,7 @@
       <c r="C142" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="D142" s="89" t="s">
+      <c r="D142" s="87" t="s">
         <v>446</v>
       </c>
       <c r="E142" s="37" t="s">
@@ -25304,7 +25334,7 @@
       <c r="C143" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="D143" s="89" t="s">
+      <c r="D143" s="87" t="s">
         <v>447</v>
       </c>
       <c r="E143" s="37" t="s">
@@ -25381,7 +25411,7 @@
       <c r="C144" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="D144" s="89" t="s">
+      <c r="D144" s="87" t="s">
         <v>448</v>
       </c>
       <c r="E144" s="37" t="s">
@@ -25458,7 +25488,7 @@
       <c r="C145" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="D145" s="89" t="s">
+      <c r="D145" s="87" t="s">
         <v>449</v>
       </c>
       <c r="E145" s="37" t="s">
@@ -25535,7 +25565,7 @@
       <c r="C146" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="D146" s="89" t="s">
+      <c r="D146" s="87" t="s">
         <v>450</v>
       </c>
       <c r="E146" s="37" t="s">
@@ -25612,7 +25642,7 @@
       <c r="C147" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="D147" s="89" t="s">
+      <c r="D147" s="87" t="s">
         <v>451</v>
       </c>
       <c r="E147" s="37" t="s">
@@ -25689,7 +25719,7 @@
       <c r="C148" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="D148" s="89" t="s">
+      <c r="D148" s="87" t="s">
         <v>452</v>
       </c>
       <c r="E148" s="37" t="s">
@@ -25766,7 +25796,7 @@
       <c r="C149" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="D149" s="89" t="s">
+      <c r="D149" s="87" t="s">
         <v>453</v>
       </c>
       <c r="E149" s="37" t="s">
@@ -25843,7 +25873,7 @@
       <c r="C150" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="D150" s="89" t="s">
+      <c r="D150" s="87" t="s">
         <v>454</v>
       </c>
       <c r="E150" s="37" t="s">
@@ -25920,7 +25950,7 @@
       <c r="C151" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="D151" s="89" t="s">
+      <c r="D151" s="87" t="s">
         <v>455</v>
       </c>
       <c r="E151" s="37" t="s">
@@ -25997,7 +26027,7 @@
       <c r="C152" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="D152" s="89" t="s">
+      <c r="D152" s="87" t="s">
         <v>456</v>
       </c>
       <c r="E152" s="37" t="s">
@@ -26074,7 +26104,7 @@
       <c r="C153" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="D153" s="89" t="s">
+      <c r="D153" s="87" t="s">
         <v>457</v>
       </c>
       <c r="E153" s="37" t="s">
@@ -26151,7 +26181,7 @@
       <c r="C154" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="D154" s="89" t="s">
+      <c r="D154" s="87" t="s">
         <v>458</v>
       </c>
       <c r="E154" s="37" t="s">
@@ -26228,7 +26258,7 @@
       <c r="C155" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="D155" s="89" t="s">
+      <c r="D155" s="87" t="s">
         <v>459</v>
       </c>
       <c r="E155" s="37" t="s">
@@ -26305,7 +26335,7 @@
       <c r="C156" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="D156" s="89" t="s">
+      <c r="D156" s="87" t="s">
         <v>460</v>
       </c>
       <c r="E156" s="37" t="s">
@@ -26382,7 +26412,7 @@
       <c r="C157" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="D157" s="89" t="s">
+      <c r="D157" s="87" t="s">
         <v>461</v>
       </c>
       <c r="E157" s="37" t="s">
@@ -26459,7 +26489,7 @@
       <c r="C158" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="D158" s="89" t="s">
+      <c r="D158" s="87" t="s">
         <v>462</v>
       </c>
       <c r="E158" s="37" t="s">
@@ -26536,7 +26566,7 @@
       <c r="C159" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="D159" s="89" t="s">
+      <c r="D159" s="87" t="s">
         <v>463</v>
       </c>
       <c r="E159" s="37" t="s">
@@ -26613,7 +26643,7 @@
       <c r="C160" s="11" t="s">
         <v>171</v>
       </c>
-      <c r="D160" s="89" t="s">
+      <c r="D160" s="87" t="s">
         <v>464</v>
       </c>
       <c r="E160" s="37" t="s">
@@ -26690,7 +26720,7 @@
       <c r="C161" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="D161" s="89" t="s">
+      <c r="D161" s="87" t="s">
         <v>465</v>
       </c>
       <c r="E161" s="37" t="s">
@@ -26767,7 +26797,7 @@
       <c r="C162" s="11" t="s">
         <v>174</v>
       </c>
-      <c r="D162" s="89" t="s">
+      <c r="D162" s="87" t="s">
         <v>466</v>
       </c>
       <c r="E162" s="37" t="s">
@@ -26844,7 +26874,7 @@
       <c r="C163" s="11" t="s">
         <v>175</v>
       </c>
-      <c r="D163" s="89" t="s">
+      <c r="D163" s="87" t="s">
         <v>467</v>
       </c>
       <c r="E163" s="37" t="s">
@@ -26921,7 +26951,7 @@
       <c r="C164" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="D164" s="87" t="s">
+      <c r="D164" s="85" t="s">
         <v>468</v>
       </c>
       <c r="E164" s="37" t="s">
@@ -26998,7 +27028,7 @@
       <c r="C165" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="D165" s="87" t="s">
+      <c r="D165" s="85" t="s">
         <v>1326</v>
       </c>
       <c r="E165" s="37" t="s">
@@ -27075,7 +27105,7 @@
       <c r="C166" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="D166" s="87" t="s">
+      <c r="D166" s="85" t="s">
         <v>470</v>
       </c>
       <c r="E166" s="37" t="s">
@@ -27152,7 +27182,7 @@
       <c r="C167" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="D167" s="87" t="s">
+      <c r="D167" s="85" t="s">
         <v>471</v>
       </c>
       <c r="E167" s="37" t="s">
@@ -27229,7 +27259,7 @@
       <c r="C168" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="D168" s="87" t="s">
+      <c r="D168" s="85" t="s">
         <v>472</v>
       </c>
       <c r="E168" s="37" t="s">
@@ -27306,7 +27336,7 @@
       <c r="C169" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="D169" s="87" t="s">
+      <c r="D169" s="85" t="s">
         <v>473</v>
       </c>
       <c r="E169" s="37" t="s">
@@ -27383,7 +27413,7 @@
       <c r="C170" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="D170" s="87" t="s">
+      <c r="D170" s="85" t="s">
         <v>474</v>
       </c>
       <c r="E170" s="37" t="s">
@@ -27460,7 +27490,7 @@
       <c r="C171" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="D171" s="90" t="s">
+      <c r="D171" s="88" t="s">
         <v>475</v>
       </c>
       <c r="E171" s="37" t="s">
@@ -27537,7 +27567,7 @@
       <c r="C172" s="11" t="s">
         <v>184</v>
       </c>
-      <c r="D172" s="91" t="s">
+      <c r="D172" s="89" t="s">
         <v>185</v>
       </c>
       <c r="E172" s="37" t="s">
@@ -27614,7 +27644,7 @@
       <c r="C173" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="D173" s="89" t="s">
+      <c r="D173" s="87" t="s">
         <v>476</v>
       </c>
       <c r="E173" s="37" t="s">
@@ -27691,7 +27721,7 @@
       <c r="C174" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="D174" s="89" t="s">
+      <c r="D174" s="87" t="s">
         <v>477</v>
       </c>
       <c r="E174" s="37" t="s">
@@ -27768,7 +27798,7 @@
       <c r="C175" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="D175" s="89" t="s">
+      <c r="D175" s="87" t="s">
         <v>478</v>
       </c>
       <c r="E175" s="37" t="s">
@@ -27845,7 +27875,7 @@
       <c r="C176" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="D176" s="90" t="s">
+      <c r="D176" s="88" t="s">
         <v>479</v>
       </c>
       <c r="E176" s="37" t="s">
@@ -27922,7 +27952,7 @@
       <c r="C177" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="D177" s="89" t="s">
+      <c r="D177" s="87" t="s">
         <v>480</v>
       </c>
       <c r="E177" s="37" t="s">
@@ -27999,7 +28029,7 @@
       <c r="C178" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="D178" s="89" t="s">
+      <c r="D178" s="87" t="s">
         <v>481</v>
       </c>
       <c r="E178" s="37" t="s">
@@ -28076,7 +28106,7 @@
       <c r="C179" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="D179" s="89" t="s">
+      <c r="D179" s="87" t="s">
         <v>482</v>
       </c>
       <c r="E179" s="37" t="s">
@@ -28153,7 +28183,7 @@
       <c r="C180" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="D180" s="89" t="s">
+      <c r="D180" s="87" t="s">
         <v>483</v>
       </c>
       <c r="E180" s="37" t="s">
@@ -28230,7 +28260,7 @@
       <c r="C181" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="D181" s="89" t="s">
+      <c r="D181" s="87" t="s">
         <v>484</v>
       </c>
       <c r="E181" s="37" t="s">
@@ -28307,7 +28337,7 @@
       <c r="C182" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="D182" s="89" t="s">
+      <c r="D182" s="87" t="s">
         <v>485</v>
       </c>
       <c r="E182" s="37" t="s">
@@ -28384,7 +28414,7 @@
       <c r="C183" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="D183" s="89" t="s">
+      <c r="D183" s="87" t="s">
         <v>486</v>
       </c>
       <c r="E183" s="37" t="s">
@@ -28461,7 +28491,7 @@
       <c r="C184" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="D184" s="89" t="s">
+      <c r="D184" s="87" t="s">
         <v>487</v>
       </c>
       <c r="E184" s="37" t="s">
@@ -28538,7 +28568,7 @@
       <c r="C185" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="D185" s="92" t="s">
+      <c r="D185" s="90" t="s">
         <v>488</v>
       </c>
       <c r="E185" s="37" t="s">
@@ -28615,7 +28645,7 @@
       <c r="C186" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="D186" s="93" t="s">
+      <c r="D186" s="91" t="s">
         <v>489</v>
       </c>
       <c r="E186" s="37" t="s">
@@ -28692,7 +28722,7 @@
       <c r="C187" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="D187" s="93" t="s">
+      <c r="D187" s="91" t="s">
         <v>490</v>
       </c>
       <c r="E187" s="37" t="s">
@@ -28769,7 +28799,7 @@
       <c r="C188" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="D188" s="93" t="s">
+      <c r="D188" s="91" t="s">
         <v>491</v>
       </c>
       <c r="E188" s="37" t="s">
@@ -28846,7 +28876,7 @@
       <c r="C189" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="D189" s="90" t="s">
+      <c r="D189" s="88" t="s">
         <v>492</v>
       </c>
       <c r="E189" s="37" t="s">
@@ -28923,7 +28953,7 @@
       <c r="C190" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="D190" s="90" t="s">
+      <c r="D190" s="88" t="s">
         <v>493</v>
       </c>
       <c r="E190" s="37" t="s">
@@ -29000,7 +29030,7 @@
       <c r="C191" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="D191" s="90" t="s">
+      <c r="D191" s="88" t="s">
         <v>494</v>
       </c>
       <c r="E191" s="37" t="s">
@@ -29077,7 +29107,7 @@
       <c r="C192" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="D192" s="90" t="s">
+      <c r="D192" s="88" t="s">
         <v>1308</v>
       </c>
       <c r="E192" s="37" t="s">
@@ -29154,7 +29184,7 @@
       <c r="C193" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="D193" s="90" t="s">
+      <c r="D193" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E193" s="37" t="s">
@@ -29231,7 +29261,7 @@
       <c r="C194" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="D194" s="90" t="s">
+      <c r="D194" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E194" s="37" t="s">
@@ -29308,7 +29338,7 @@
       <c r="C195" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="D195" s="90" t="s">
+      <c r="D195" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E195" s="37" t="s">
@@ -29385,7 +29415,7 @@
       <c r="C196" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="D196" s="90" t="s">
+      <c r="D196" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E196" s="37" t="s">
@@ -29462,7 +29492,7 @@
       <c r="C197" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="D197" s="90" t="s">
+      <c r="D197" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E197" s="37" t="s">
@@ -29539,7 +29569,7 @@
       <c r="C198" s="11" t="s">
         <v>214</v>
       </c>
-      <c r="D198" s="90" t="s">
+      <c r="D198" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E198" s="37" t="s">
@@ -29616,7 +29646,7 @@
       <c r="C199" s="11" t="s">
         <v>215</v>
       </c>
-      <c r="D199" s="90" t="s">
+      <c r="D199" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E199" s="37" t="s">
@@ -29693,7 +29723,7 @@
       <c r="C200" s="11" t="s">
         <v>216</v>
       </c>
-      <c r="D200" s="90" t="s">
+      <c r="D200" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E200" s="37" t="s">
@@ -29751,7 +29781,7 @@
         <v>1559</v>
       </c>
       <c r="W200" s="18" t="str">
-        <f t="shared" ref="W200:W225" si="8">CONCATENATE("['",B200,"', '",C200,"', '",D200,"', '",E200,"', ",F200,", ",G200,", ",H200,", ",I200,", ",J200,", ",K200,", '",L200,"', ",M200,", ",N200,", ",O200,", ",P200,", ",Q200,", ",R200,", ",S200,", ",T200,"], ")</f>
+        <f t="shared" ref="W200:W229" si="8">CONCATENATE("['",B200,"', '",C200,"', '",D200,"', '",E200,"', ",F200,", ",G200,", ",H200,", ",I200,", ",J200,", ",K200,", '",L200,"', ",M200,", ",N200,", ",O200,", ",P200,", ",Q200,", ",R200,", ",S200,", ",T200,"], ")</f>
         <v xml:space="preserve">['A107', 'A107', 'OTRO', 'Pza.', 0, 0, 0, 0, 0, 0, 'ALVICRUZ - cbba -  -  - santa puej -  - ', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
       <c r="X200" s="18"/>
@@ -29770,7 +29800,7 @@
       <c r="C201" s="11" t="s">
         <v>217</v>
       </c>
-      <c r="D201" s="90" t="s">
+      <c r="D201" s="88" t="s">
         <v>1304</v>
       </c>
       <c r="E201" s="37" t="s">
@@ -29847,7 +29877,7 @@
       <c r="C202" s="78" t="s">
         <v>1284</v>
       </c>
-      <c r="D202" s="94" t="s">
+      <c r="D202" s="92" t="s">
         <v>1290</v>
       </c>
       <c r="E202" s="79" t="s">
@@ -29920,7 +29950,7 @@
       <c r="C203" s="78" t="s">
         <v>1285</v>
       </c>
-      <c r="D203" s="94" t="s">
+      <c r="D203" s="92" t="s">
         <v>1356</v>
       </c>
       <c r="E203" s="79" t="s">
@@ -29993,7 +30023,7 @@
       <c r="C204" s="78" t="s">
         <v>1286</v>
       </c>
-      <c r="D204" s="94" t="s">
+      <c r="D204" s="92" t="s">
         <v>1291</v>
       </c>
       <c r="E204" s="79" t="s">
@@ -30066,7 +30096,7 @@
       <c r="C205" s="78" t="s">
         <v>1287</v>
       </c>
-      <c r="D205" s="94" t="s">
+      <c r="D205" s="92" t="s">
         <v>1292</v>
       </c>
       <c r="E205" s="79" t="s">
@@ -30139,7 +30169,7 @@
       <c r="C206" s="78" t="s">
         <v>1288</v>
       </c>
-      <c r="D206" s="94" t="s">
+      <c r="D206" s="92" t="s">
         <v>1293</v>
       </c>
       <c r="E206" s="79" t="s">
@@ -30212,7 +30242,7 @@
       <c r="C207" s="78" t="s">
         <v>1289</v>
       </c>
-      <c r="D207" s="94" t="s">
+      <c r="D207" s="92" t="s">
         <v>1294</v>
       </c>
       <c r="E207" s="79" t="s">
@@ -30285,7 +30315,7 @@
       <c r="C208" s="78" t="s">
         <v>1338</v>
       </c>
-      <c r="D208" s="94" t="s">
+      <c r="D208" s="92" t="s">
         <v>1295</v>
       </c>
       <c r="E208" s="37" t="s">
@@ -30354,7 +30384,7 @@
       <c r="C209" s="78" t="s">
         <v>1339</v>
       </c>
-      <c r="D209" s="94" t="s">
+      <c r="D209" s="92" t="s">
         <v>1296</v>
       </c>
       <c r="E209" s="37" t="s">
@@ -30423,7 +30453,7 @@
       <c r="C210" s="78" t="s">
         <v>1340</v>
       </c>
-      <c r="D210" s="94" t="s">
+      <c r="D210" s="92" t="s">
         <v>1297</v>
       </c>
       <c r="E210" s="37" t="s">
@@ -30492,7 +30522,7 @@
       <c r="C211" s="78" t="s">
         <v>1341</v>
       </c>
-      <c r="D211" s="94" t="s">
+      <c r="D211" s="92" t="s">
         <v>1298</v>
       </c>
       <c r="E211" s="37" t="s">
@@ -30556,13 +30586,13 @@
         <v>206</v>
       </c>
       <c r="B212" s="78" t="s">
-        <v>1342</v>
+        <v>1575</v>
       </c>
       <c r="C212" s="78" t="s">
-        <v>1342</v>
-      </c>
-      <c r="D212" s="94" t="s">
-        <v>1309</v>
+        <v>1575</v>
+      </c>
+      <c r="D212" s="92" t="s">
+        <v>1577</v>
       </c>
       <c r="E212" s="37" t="s">
         <v>1302</v>
@@ -30613,11 +30643,11 @@
         <v>0</v>
       </c>
       <c r="V212" s="6" t="s">
-        <v>1565</v>
+        <v>1585</v>
       </c>
       <c r="W212" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">['FTTS10', 'FTTS10', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f>CONCATENATE("['",B212,"', '",C212,"', '",D212,"', '",E212,"', ",F212,", ",G212,", ",H212,", ",I212,", ",J212,", ",K212,", '",L212,"', ",M212,", ",N212,", ",O212,", ",P212,", ",Q212,", ",R212,", ",S212,", ",T212,"], ")</f>
+        <v xml:space="preserve">['FTCV8', 'FTCV8', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="213" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30625,13 +30655,13 @@
         <v>207</v>
       </c>
       <c r="B213" s="78" t="s">
-        <v>1343</v>
+        <v>1576</v>
       </c>
       <c r="C213" s="78" t="s">
-        <v>1343</v>
-      </c>
-      <c r="D213" s="94" t="s">
-        <v>1310</v>
+        <v>1576</v>
+      </c>
+      <c r="D213" s="92" t="s">
+        <v>1578</v>
       </c>
       <c r="E213" s="37" t="s">
         <v>1302</v>
@@ -30682,11 +30712,11 @@
         <v>0</v>
       </c>
       <c r="V213" s="6" t="s">
-        <v>1566</v>
+        <v>1586</v>
       </c>
       <c r="W213" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">['FTTS10C', 'FTTS10C', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f>CONCATENATE("['",B213,"', '",C213,"', '",D213,"', '",E213,"', ",F213,", ",G213,", ",H213,", ",I213,", ",J213,", ",K213,", '",L213,"', ",M213,", ",N213,", ",O213,", ",P213,", ",Q213,", ",R213,", ",S213,", ",T213,"], ")</f>
+        <v xml:space="preserve">['FTCV8C', 'FTCV8C', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="214" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30694,13 +30724,13 @@
         <v>208</v>
       </c>
       <c r="B214" s="78" t="s">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="C214" s="78" t="s">
-        <v>1344</v>
-      </c>
-      <c r="D214" s="94" t="s">
-        <v>1311</v>
+        <v>1342</v>
+      </c>
+      <c r="D214" s="92" t="s">
+        <v>1309</v>
       </c>
       <c r="E214" s="37" t="s">
         <v>1302</v>
@@ -30751,11 +30781,11 @@
         <v>0</v>
       </c>
       <c r="V214" s="6" t="s">
-        <v>1567</v>
+        <v>1587</v>
       </c>
       <c r="W214" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['FTCV10', 'FTCV10', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['FTTS10', 'FTTS10', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="215" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30763,13 +30793,13 @@
         <v>209</v>
       </c>
       <c r="B215" s="78" t="s">
-        <v>1345</v>
+        <v>1343</v>
       </c>
       <c r="C215" s="78" t="s">
-        <v>1345</v>
-      </c>
-      <c r="D215" s="94" t="s">
-        <v>1312</v>
+        <v>1343</v>
+      </c>
+      <c r="D215" s="92" t="s">
+        <v>1310</v>
       </c>
       <c r="E215" s="37" t="s">
         <v>1302</v>
@@ -30820,11 +30850,11 @@
         <v>0</v>
       </c>
       <c r="V215" s="6" t="s">
-        <v>1568</v>
+        <v>1588</v>
       </c>
       <c r="W215" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['FTCV10C', 'FTCV10C', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['FTTS10C', 'FTTS10C', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="216" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30832,13 +30862,13 @@
         <v>210</v>
       </c>
       <c r="B216" s="78" t="s">
-        <v>1346</v>
+        <v>1575</v>
       </c>
       <c r="C216" s="78" t="s">
-        <v>1346</v>
-      </c>
-      <c r="D216" s="94" t="s">
-        <v>1313</v>
+        <v>1575</v>
+      </c>
+      <c r="D216" s="92" t="s">
+        <v>1573</v>
       </c>
       <c r="E216" s="37" t="s">
         <v>1302</v>
@@ -30889,11 +30919,11 @@
         <v>0</v>
       </c>
       <c r="V216" s="6" t="s">
-        <v>1569</v>
+        <v>1589</v>
       </c>
       <c r="W216" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['VC2H8', 'VC2H8', 'VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['FTCV8', 'FTCV8', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="217" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30901,13 +30931,13 @@
         <v>211</v>
       </c>
       <c r="B217" s="78" t="s">
-        <v>1347</v>
+        <v>1576</v>
       </c>
       <c r="C217" s="78" t="s">
-        <v>1347</v>
-      </c>
-      <c r="D217" s="94" t="s">
-        <v>1314</v>
+        <v>1576</v>
+      </c>
+      <c r="D217" s="92" t="s">
+        <v>1574</v>
       </c>
       <c r="E217" s="37" t="s">
         <v>1302</v>
@@ -30958,11 +30988,11 @@
         <v>0</v>
       </c>
       <c r="V217" s="6" t="s">
-        <v>1570</v>
+        <v>1590</v>
       </c>
       <c r="W217" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['VC2H8C', 'VC2H8C', 'VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['FTCV8C', 'FTCV8C', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="218" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30970,13 +31000,13 @@
         <v>212</v>
       </c>
       <c r="B218" s="78" t="s">
-        <v>1348</v>
+        <v>1344</v>
       </c>
       <c r="C218" s="78" t="s">
-        <v>1348</v>
-      </c>
-      <c r="D218" s="94" t="s">
-        <v>1315</v>
+        <v>1344</v>
+      </c>
+      <c r="D218" s="92" t="s">
+        <v>1311</v>
       </c>
       <c r="E218" s="37" t="s">
         <v>1302</v>
@@ -31027,11 +31057,11 @@
         <v>0</v>
       </c>
       <c r="V218" s="6" t="s">
-        <v>1571</v>
+        <v>1591</v>
       </c>
       <c r="W218" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">['VC4H8', 'VC4H8', 'VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f t="shared" ref="W218:W219" si="9">CONCATENATE("['",B218,"', '",C218,"', '",D218,"', '",E218,"', ",F218,", ",G218,", ",H218,", ",I218,", ",J218,", ",K218,", '",L218,"', ",M218,", ",N218,", ",O218,", ",P218,", ",Q218,", ",R218,", ",S218,", ",T218,"], ")</f>
+        <v xml:space="preserve">['FTCV10', 'FTCV10', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="219" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31039,13 +31069,13 @@
         <v>213</v>
       </c>
       <c r="B219" s="78" t="s">
-        <v>1349</v>
+        <v>1345</v>
       </c>
       <c r="C219" s="78" t="s">
-        <v>1349</v>
-      </c>
-      <c r="D219" s="94" t="s">
-        <v>1316</v>
+        <v>1345</v>
+      </c>
+      <c r="D219" s="92" t="s">
+        <v>1312</v>
       </c>
       <c r="E219" s="37" t="s">
         <v>1302</v>
@@ -31096,11 +31126,11 @@
         <v>0</v>
       </c>
       <c r="V219" s="6" t="s">
-        <v>1572</v>
+        <v>1592</v>
       </c>
       <c r="W219" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">['VC4H8C', 'VC4H8C', 'VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve">['FTCV10C', 'FTCV10C', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="220" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31108,13 +31138,13 @@
         <v>214</v>
       </c>
       <c r="B220" s="78" t="s">
-        <v>1350</v>
+        <v>1346</v>
       </c>
       <c r="C220" s="78" t="s">
-        <v>1350</v>
-      </c>
-      <c r="D220" s="94" t="s">
-        <v>1317</v>
+        <v>1346</v>
+      </c>
+      <c r="D220" s="92" t="s">
+        <v>1313</v>
       </c>
       <c r="E220" s="37" t="s">
         <v>1302</v>
@@ -31165,11 +31195,11 @@
         <v>0</v>
       </c>
       <c r="V220" s="6" t="s">
-        <v>1573</v>
+        <v>1593</v>
       </c>
       <c r="W220" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PVC2H10', 'PVC2H10', 'PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['VC2H8', 'VC2H8', 'VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="221" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31177,13 +31207,13 @@
         <v>215</v>
       </c>
       <c r="B221" s="78" t="s">
-        <v>1351</v>
+        <v>1347</v>
       </c>
       <c r="C221" s="78" t="s">
-        <v>1351</v>
-      </c>
-      <c r="D221" s="94" t="s">
-        <v>1318</v>
+        <v>1347</v>
+      </c>
+      <c r="D221" s="92" t="s">
+        <v>1314</v>
       </c>
       <c r="E221" s="37" t="s">
         <v>1302</v>
@@ -31234,11 +31264,11 @@
         <v>0</v>
       </c>
       <c r="V221" s="6" t="s">
-        <v>1574</v>
+        <v>1594</v>
       </c>
       <c r="W221" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PVC2H10C', 'PVC2H10C', 'PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['VC2H8C', 'VC2H8C', 'VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="222" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31246,13 +31276,13 @@
         <v>216</v>
       </c>
       <c r="B222" s="78" t="s">
-        <v>1352</v>
+        <v>1348</v>
       </c>
       <c r="C222" s="78" t="s">
-        <v>1352</v>
-      </c>
-      <c r="D222" s="94" t="s">
-        <v>1319</v>
+        <v>1348</v>
+      </c>
+      <c r="D222" s="92" t="s">
+        <v>1315</v>
       </c>
       <c r="E222" s="37" t="s">
         <v>1302</v>
@@ -31303,11 +31333,11 @@
         <v>0</v>
       </c>
       <c r="V222" s="6" t="s">
-        <v>1575</v>
+        <v>1595</v>
       </c>
       <c r="W222" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PVC4H10', 'PVC4H10', 'PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['VC4H8', 'VC4H8', 'VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="223" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31315,13 +31345,13 @@
         <v>217</v>
       </c>
       <c r="B223" s="78" t="s">
-        <v>1353</v>
+        <v>1349</v>
       </c>
       <c r="C223" s="78" t="s">
-        <v>1353</v>
-      </c>
-      <c r="D223" s="94" t="s">
-        <v>1320</v>
+        <v>1349</v>
+      </c>
+      <c r="D223" s="92" t="s">
+        <v>1316</v>
       </c>
       <c r="E223" s="37" t="s">
         <v>1302</v>
@@ -31372,11 +31402,11 @@
         <v>0</v>
       </c>
       <c r="V223" s="6" t="s">
-        <v>1576</v>
+        <v>1596</v>
       </c>
       <c r="W223" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PVC4H10C', 'PVC4H10C', 'PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['VC4H8C', 'VC4H8C', 'VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="224" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31384,13 +31414,13 @@
         <v>218</v>
       </c>
       <c r="B224" s="78" t="s">
-        <v>1354</v>
+        <v>1350</v>
       </c>
       <c r="C224" s="78" t="s">
-        <v>1354</v>
-      </c>
-      <c r="D224" s="94" t="s">
-        <v>1587</v>
+        <v>1350</v>
+      </c>
+      <c r="D224" s="92" t="s">
+        <v>1317</v>
       </c>
       <c r="E224" s="37" t="s">
         <v>1302</v>
@@ -31441,11 +31471,11 @@
         <v>0</v>
       </c>
       <c r="V224" s="6" t="s">
-        <v>1577</v>
+        <v>1597</v>
       </c>
       <c r="W224" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PB10', 'PB10', 'PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PVC2H10', 'PVC2H10', 'PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="225" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31453,13 +31483,13 @@
         <v>219</v>
       </c>
       <c r="B225" s="78" t="s">
-        <v>1355</v>
+        <v>1351</v>
       </c>
       <c r="C225" s="78" t="s">
-        <v>1355</v>
-      </c>
-      <c r="D225" s="94" t="s">
-        <v>1588</v>
+        <v>1351</v>
+      </c>
+      <c r="D225" s="92" t="s">
+        <v>1318</v>
       </c>
       <c r="E225" s="37" t="s">
         <v>1302</v>
@@ -31510,11 +31540,11 @@
         <v>0</v>
       </c>
       <c r="V225" s="6" t="s">
-        <v>1578</v>
+        <v>1598</v>
       </c>
       <c r="W225" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PB10C', 'PB10C', 'PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PVC2H10C', 'PVC2H10C', 'PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="226" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31522,13 +31552,13 @@
         <v>220</v>
       </c>
       <c r="B226" s="78" t="s">
-        <v>1585</v>
+        <v>1352</v>
       </c>
       <c r="C226" s="78" t="s">
-        <v>1585</v>
-      </c>
-      <c r="D226" s="94" t="s">
-        <v>1589</v>
+        <v>1352</v>
+      </c>
+      <c r="D226" s="92" t="s">
+        <v>1319</v>
       </c>
       <c r="E226" s="37" t="s">
         <v>1302</v>
@@ -31579,11 +31609,11 @@
         <v>0</v>
       </c>
       <c r="V226" s="6" t="s">
-        <v>1591</v>
+        <v>1599</v>
       </c>
       <c r="W226" s="18" t="str">
-        <f t="shared" ref="W226:W227" si="9">CONCATENATE("['",B226,"', '",C226,"', '",D226,"', '",E226,"', ",F226,", ",G226,", ",H226,", ",I226,", ",J226,", ",K226,", '",L226,"', ",M226,", ",N226,", ",O226,", ",P226,", ",Q226,", ",R226,", ",S226,", ",T226,"], ")</f>
-        <v xml:space="preserve">['PB10CF', 'PB10CF', 'PUERTAS BATIENTES CON FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">['PVC4H10', 'PVC4H10', 'PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="227" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31591,13 +31621,13 @@
         <v>221</v>
       </c>
       <c r="B227" s="78" t="s">
-        <v>1586</v>
+        <v>1353</v>
       </c>
       <c r="C227" s="78" t="s">
-        <v>1586</v>
-      </c>
-      <c r="D227" s="94" t="s">
-        <v>1590</v>
+        <v>1353</v>
+      </c>
+      <c r="D227" s="92" t="s">
+        <v>1320</v>
       </c>
       <c r="E227" s="37" t="s">
         <v>1302</v>
@@ -31648,10 +31678,286 @@
         <v>0</v>
       </c>
       <c r="V227" s="6" t="s">
-        <v>1592</v>
+        <v>1600</v>
       </c>
       <c r="W227" s="18" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">['PVC4H10C', 'PVC4H10C', 'PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+      </c>
+    </row>
+    <row r="228" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A228" s="77">
+        <v>222</v>
+      </c>
+      <c r="B228" s="78" t="s">
+        <v>1354</v>
+      </c>
+      <c r="C228" s="78" t="s">
+        <v>1354</v>
+      </c>
+      <c r="D228" s="92" t="s">
+        <v>1567</v>
+      </c>
+      <c r="E228" s="37" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F228" s="10">
+        <v>0</v>
+      </c>
+      <c r="G228" s="10">
+        <v>0</v>
+      </c>
+      <c r="H228" s="60">
+        <v>0</v>
+      </c>
+      <c r="I228" s="60">
+        <v>0</v>
+      </c>
+      <c r="J228" s="60">
+        <v>0</v>
+      </c>
+      <c r="K228" s="60">
+        <v>0</v>
+      </c>
+      <c r="L228" s="60" t="s">
+        <v>1303</v>
+      </c>
+      <c r="M228" s="60">
+        <v>0</v>
+      </c>
+      <c r="N228" s="60">
+        <v>0</v>
+      </c>
+      <c r="O228" s="60">
+        <v>0</v>
+      </c>
+      <c r="P228" s="60">
+        <v>0</v>
+      </c>
+      <c r="Q228" s="60">
+        <v>0</v>
+      </c>
+      <c r="R228" s="60">
+        <v>0</v>
+      </c>
+      <c r="S228" s="60">
+        <v>0</v>
+      </c>
+      <c r="T228" s="60">
+        <v>0</v>
+      </c>
+      <c r="V228" s="6" t="s">
+        <v>1601</v>
+      </c>
+      <c r="W228" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">['PB10', 'PB10', 'PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+      </c>
+    </row>
+    <row r="229" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A229" s="77">
+        <v>223</v>
+      </c>
+      <c r="B229" s="78" t="s">
+        <v>1355</v>
+      </c>
+      <c r="C229" s="78" t="s">
+        <v>1355</v>
+      </c>
+      <c r="D229" s="92" t="s">
+        <v>1568</v>
+      </c>
+      <c r="E229" s="37" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F229" s="10">
+        <v>0</v>
+      </c>
+      <c r="G229" s="10">
+        <v>0</v>
+      </c>
+      <c r="H229" s="60">
+        <v>0</v>
+      </c>
+      <c r="I229" s="60">
+        <v>0</v>
+      </c>
+      <c r="J229" s="60">
+        <v>0</v>
+      </c>
+      <c r="K229" s="60">
+        <v>0</v>
+      </c>
+      <c r="L229" s="60" t="s">
+        <v>1303</v>
+      </c>
+      <c r="M229" s="60">
+        <v>0</v>
+      </c>
+      <c r="N229" s="60">
+        <v>0</v>
+      </c>
+      <c r="O229" s="60">
+        <v>0</v>
+      </c>
+      <c r="P229" s="60">
+        <v>0</v>
+      </c>
+      <c r="Q229" s="60">
+        <v>0</v>
+      </c>
+      <c r="R229" s="60">
+        <v>0</v>
+      </c>
+      <c r="S229" s="60">
+        <v>0</v>
+      </c>
+      <c r="T229" s="60">
+        <v>0</v>
+      </c>
+      <c r="V229" s="6" t="s">
+        <v>1602</v>
+      </c>
+      <c r="W229" s="18" t="str">
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">['PB10C', 'PB10C', 'PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+      </c>
+    </row>
+    <row r="230" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A230" s="77">
+        <v>224</v>
+      </c>
+      <c r="B230" s="78" t="s">
+        <v>1565</v>
+      </c>
+      <c r="C230" s="78" t="s">
+        <v>1565</v>
+      </c>
+      <c r="D230" s="92" t="s">
+        <v>1569</v>
+      </c>
+      <c r="E230" s="37" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F230" s="10">
+        <v>0</v>
+      </c>
+      <c r="G230" s="10">
+        <v>0</v>
+      </c>
+      <c r="H230" s="60">
+        <v>0</v>
+      </c>
+      <c r="I230" s="60">
+        <v>0</v>
+      </c>
+      <c r="J230" s="60">
+        <v>0</v>
+      </c>
+      <c r="K230" s="60">
+        <v>0</v>
+      </c>
+      <c r="L230" s="60" t="s">
+        <v>1303</v>
+      </c>
+      <c r="M230" s="60">
+        <v>0</v>
+      </c>
+      <c r="N230" s="60">
+        <v>0</v>
+      </c>
+      <c r="O230" s="60">
+        <v>0</v>
+      </c>
+      <c r="P230" s="60">
+        <v>0</v>
+      </c>
+      <c r="Q230" s="60">
+        <v>0</v>
+      </c>
+      <c r="R230" s="60">
+        <v>0</v>
+      </c>
+      <c r="S230" s="60">
+        <v>0</v>
+      </c>
+      <c r="T230" s="60">
+        <v>0</v>
+      </c>
+      <c r="V230" s="6" t="s">
+        <v>1571</v>
+      </c>
+      <c r="W230" s="18" t="str">
+        <f t="shared" ref="W230:W231" si="10">CONCATENATE("['",B230,"', '",C230,"', '",D230,"', '",E230,"', ",F230,", ",G230,", ",H230,", ",I230,", ",J230,", ",K230,", '",L230,"', ",M230,", ",N230,", ",O230,", ",P230,", ",Q230,", ",R230,", ",S230,", ",T230,"], ")</f>
+        <v xml:space="preserve">['PB10CF', 'PB10CF', 'PUERTAS BATIENTES CON FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+      </c>
+    </row>
+    <row r="231" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A231" s="77">
+        <v>225</v>
+      </c>
+      <c r="B231" s="78" t="s">
+        <v>1566</v>
+      </c>
+      <c r="C231" s="78" t="s">
+        <v>1566</v>
+      </c>
+      <c r="D231" s="92" t="s">
+        <v>1570</v>
+      </c>
+      <c r="E231" s="37" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F231" s="10">
+        <v>0</v>
+      </c>
+      <c r="G231" s="10">
+        <v>0</v>
+      </c>
+      <c r="H231" s="60">
+        <v>0</v>
+      </c>
+      <c r="I231" s="60">
+        <v>0</v>
+      </c>
+      <c r="J231" s="60">
+        <v>0</v>
+      </c>
+      <c r="K231" s="60">
+        <v>0</v>
+      </c>
+      <c r="L231" s="60" t="s">
+        <v>1303</v>
+      </c>
+      <c r="M231" s="60">
+        <v>0</v>
+      </c>
+      <c r="N231" s="60">
+        <v>0</v>
+      </c>
+      <c r="O231" s="60">
+        <v>0</v>
+      </c>
+      <c r="P231" s="60">
+        <v>0</v>
+      </c>
+      <c r="Q231" s="60">
+        <v>0</v>
+      </c>
+      <c r="R231" s="60">
+        <v>0</v>
+      </c>
+      <c r="S231" s="60">
+        <v>0</v>
+      </c>
+      <c r="T231" s="60">
+        <v>0</v>
+      </c>
+      <c r="V231" s="6" t="s">
+        <v>1572</v>
+      </c>
+      <c r="W231" s="18" t="str">
+        <f t="shared" si="10"/>
         <v xml:space="preserve">['PB10CFC', 'PB10CFC', 'PUERTAS BATIENTES CON FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>

</xml_diff>

<commit_message>
avanzando en la interfaz y control de errores
</commit_message>
<xml_diff>
--- a/TRABAJOS-PYTHON/COTIZA_ALU_TEM/lista_materiales.xlsx
+++ b/TRABAJOS-PYTHON/COTIZA_ALU_TEM/lista_materiales.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PcAsusZenbookRafita\Desktop\REPO_RAFAEL_ANTEQUERA\TRABAJOS-PYTHON\COTIZA_ALU_TEM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{613BABF8-3F63-4605-80AB-CEFB34171A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD0F240-1506-4C1B-92E6-1601C1B6F9F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{1B3D5D76-0D2B-4247-8E51-F5AC57810600}"/>
   </bookViews>
@@ -18,10 +18,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Costo M.P.yMat.'!$A$2:$F$94</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Costo M.P.yMat. (2)'!$A$2:$T$231</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Costo M.P.yMat. (2)'!$A$2:$T$232</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Costo M.P.yMat. (2)'!$2:$5</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3596" uniqueCount="1603">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3616" uniqueCount="1605">
   <si>
     <t>ANALISIS DE COSTOS Y DETERMINACION DE PRECIOS DE VENTA (/i1,1/,84)</t>
   </si>
@@ -4849,13 +4849,19 @@
   </si>
   <si>
     <t xml:space="preserve">["PB10C", "PB10C", "PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ", "Pza(s).", 0, 0, 0, 0, 0, 0, "Datos para proforma", 0, 0, 0, 0, 0, 0, 0, 0], </t>
+  </si>
+  <si>
+    <t>TECNICO</t>
+  </si>
+  <si>
+    <t>TEC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -4936,6 +4942,13 @@
       <u/>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
+      <name val="Rockwell"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="12"/>
       <name val="Rockwell"/>
       <family val="1"/>
     </font>
@@ -5155,7 +5168,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
@@ -5387,6 +5400,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -14545,7 +14561,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB231"/>
+  <dimension ref="A1:AB232"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="27.6" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="72" customWidth="1"/>
@@ -24319,7 +24335,7 @@
       </c>
       <c r="X129" s="18"/>
       <c r="AB129" s="1" t="str">
-        <f t="shared" ref="AB129:AB207" si="5">CONCATENATE("['",B129,"', '",C129,"', '",D129,"', ",0,", '",E129,"'],")</f>
+        <f t="shared" ref="AB129:AB208" si="5">CONCATENATE("['",B129,"', '",C129,"', '",D129,"', ",0,", '",E129,"'],")</f>
         <v>['A36', 'A36', 'CELOSIAS 3 ALETAS - 460 MM.', 0, 'Par'],</v>
       </c>
     </row>
@@ -29170,7 +29186,7 @@
       </c>
       <c r="X192" s="18"/>
       <c r="AB192" s="1" t="str">
-        <f t="shared" ref="AB192:AB201" si="7">CONCATENATE("['",B192,"', '",C192,"', '",D192,"', ",0,", '",E192,"'],")</f>
+        <f t="shared" ref="AB192:AB202" si="7">CONCATENATE("['",B192,"', '",C192,"', '",D192,"', ",0,", '",E192,"'],")</f>
         <v>['A99', 'A99', 'ESMERILADO', 0, 'Pza.'],</v>
       </c>
     </row>
@@ -29781,7 +29797,7 @@
         <v>1559</v>
       </c>
       <c r="W200" s="18" t="str">
-        <f t="shared" ref="W200:W229" si="8">CONCATENATE("['",B200,"', '",C200,"', '",D200,"', '",E200,"', ",F200,", ",G200,", ",H200,", ",I200,", ",J200,", ",K200,", '",L200,"', ",M200,", ",N200,", ",O200,", ",P200,", ",Q200,", ",R200,", ",S200,", ",T200,"], ")</f>
+        <f t="shared" ref="W200:W230" si="8">CONCATENATE("['",B200,"', '",C200,"', '",D200,"', '",E200,"', ",F200,", ",G200,", ",H200,", ",I200,", ",J200,", ",K200,", '",L200,"', ",M200,", ",N200,", ",O200,", ",P200,", ",Q200,", ",R200,", ",S200,", ",T200,"], ")</f>
         <v xml:space="preserve">['A107', 'A107', 'OTRO', 'Pza.', 0, 0, 0, 0, 0, 0, 'ALVICRUZ - cbba -  -  - santa puej -  - ', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
       <c r="X200" s="18"/>
@@ -29872,13 +29888,13 @@
         <v>196</v>
       </c>
       <c r="B202" s="78" t="s">
-        <v>1284</v>
+        <v>1604</v>
       </c>
       <c r="C202" s="78" t="s">
-        <v>1284</v>
-      </c>
-      <c r="D202" s="92" t="s">
-        <v>1290</v>
+        <v>1604</v>
+      </c>
+      <c r="D202" s="96" t="s">
+        <v>1603</v>
       </c>
       <c r="E202" s="79" t="s">
         <v>1359</v>
@@ -29932,12 +29948,12 @@
         <v>1579</v>
       </c>
       <c r="W202" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">['OB', 'OB', 'OBRA  ', 'obra',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
+        <f t="shared" ref="W202" si="9">CONCATENATE("['",B202,"', '",C202,"', '",D202,"', '",E202,"', ",F202,", ",G202,", ",H202,", ",I202,", ",J202,", ",K202,", '",L202,"', ",M202,", ",N202,", ",O202,", ",P202,", ",Q202,", ",R202,", ",S202,", ",T202,"], ")</f>
+        <v xml:space="preserve">['TEC', 'TEC', 'TECNICO', 'obra',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
       </c>
       <c r="AB202" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>['OB', 'OB', 'OBRA  ', 0, 'obra'],</v>
+        <f t="shared" si="7"/>
+        <v>['TEC', 'TEC', 'TECNICO', 0, 'obra'],</v>
       </c>
     </row>
     <row r="203" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
@@ -29945,16 +29961,16 @@
         <v>197</v>
       </c>
       <c r="B203" s="78" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="C203" s="78" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="D203" s="92" t="s">
-        <v>1356</v>
+        <v>1290</v>
       </c>
       <c r="E203" s="79" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="F203" s="79" t="s">
         <v>495</v>
@@ -30002,15 +30018,15 @@
         <v>495</v>
       </c>
       <c r="V203" s="6" t="s">
-        <v>1580</v>
+        <v>1579</v>
       </c>
       <c r="W203" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['CL', 'CL', 'CLIENTE  ', 'cliente',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
+        <v xml:space="preserve">['OB', 'OB', 'OBRA  ', 'obra',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
       </c>
       <c r="AB203" s="1" t="str">
         <f t="shared" si="5"/>
-        <v>['CL', 'CL', 'CLIENTE  ', 0, 'cliente'],</v>
+        <v>['OB', 'OB', 'OBRA  ', 0, 'obra'],</v>
       </c>
     </row>
     <row r="204" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
@@ -30018,16 +30034,16 @@
         <v>198</v>
       </c>
       <c r="B204" s="78" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="C204" s="78" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="D204" s="92" t="s">
-        <v>1291</v>
+        <v>1356</v>
       </c>
       <c r="E204" s="79" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
       <c r="F204" s="79" t="s">
         <v>495</v>
@@ -30075,15 +30091,15 @@
         <v>495</v>
       </c>
       <c r="V204" s="6" t="s">
-        <v>1581</v>
+        <v>1580</v>
       </c>
       <c r="W204" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['TE', 'TE', 'TELEFONO  ', 'telefono',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
+        <v xml:space="preserve">['CL', 'CL', 'CLIENTE  ', 'cliente',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
       </c>
       <c r="AB204" s="1" t="str">
         <f t="shared" si="5"/>
-        <v>['TE', 'TE', 'TELEFONO  ', 0, 'telefono'],</v>
+        <v>['CL', 'CL', 'CLIENTE  ', 0, 'cliente'],</v>
       </c>
     </row>
     <row r="205" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
@@ -30091,16 +30107,16 @@
         <v>199</v>
       </c>
       <c r="B205" s="78" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="C205" s="78" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="D205" s="92" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="E205" s="79" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="F205" s="79" t="s">
         <v>495</v>
@@ -30148,15 +30164,15 @@
         <v>495</v>
       </c>
       <c r="V205" s="6" t="s">
-        <v>1582</v>
+        <v>1581</v>
       </c>
       <c r="W205" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['DI', 'DI', 'DIRECCION  ', 'direccion',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
+        <v xml:space="preserve">['TE', 'TE', 'TELEFONO  ', 'telefono',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
       </c>
       <c r="AB205" s="1" t="str">
         <f t="shared" si="5"/>
-        <v>['DI', 'DI', 'DIRECCION  ', 0, 'direccion'],</v>
+        <v>['TE', 'TE', 'TELEFONO  ', 0, 'telefono'],</v>
       </c>
     </row>
     <row r="206" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
@@ -30164,16 +30180,16 @@
         <v>200</v>
       </c>
       <c r="B206" s="78" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="C206" s="78" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="D206" s="92" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="E206" s="79" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="F206" s="79" t="s">
         <v>495</v>
@@ -30221,15 +30237,15 @@
         <v>495</v>
       </c>
       <c r="V206" s="6" t="s">
-        <v>1583</v>
+        <v>1582</v>
       </c>
       <c r="W206" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['CO', 'CO', 'CORREO  ', 'correo',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
+        <v xml:space="preserve">['DI', 'DI', 'DIRECCION  ', 'direccion',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
       </c>
       <c r="AB206" s="1" t="str">
         <f t="shared" si="5"/>
-        <v>['CO', 'CO', 'CORREO  ', 0, 'correo'],</v>
+        <v>['DI', 'DI', 'DIRECCION  ', 0, 'direccion'],</v>
       </c>
     </row>
     <row r="207" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
@@ -30237,16 +30253,16 @@
         <v>201</v>
       </c>
       <c r="B207" s="78" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="C207" s="78" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D207" s="92" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="E207" s="79" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="F207" s="79" t="s">
         <v>495</v>
@@ -30294,84 +30310,88 @@
         <v>495</v>
       </c>
       <c r="V207" s="6" t="s">
-        <v>1584</v>
+        <v>1583</v>
       </c>
       <c r="W207" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['OBS', 'OBS', 'OBSERVACIONES  ', 'observa',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
+        <v xml:space="preserve">['CO', 'CO', 'CORREO  ', 'correo',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
       </c>
       <c r="AB207" s="1" t="str">
         <f t="shared" si="5"/>
-        <v>['OBS', 'OBS', 'OBSERVACIONES  ', 0, 'observa'],</v>
-      </c>
-    </row>
-    <row r="208" spans="1:28" ht="31.2" x14ac:dyDescent="0.3">
+        <v>['CO', 'CO', 'CORREO  ', 0, 'correo'],</v>
+      </c>
+    </row>
+    <row r="208" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A208" s="77">
         <v>202</v>
       </c>
       <c r="B208" s="78" t="s">
-        <v>1338</v>
+        <v>1289</v>
       </c>
       <c r="C208" s="78" t="s">
-        <v>1338</v>
+        <v>1289</v>
       </c>
       <c r="D208" s="92" t="s">
-        <v>1295</v>
-      </c>
-      <c r="E208" s="37" t="s">
-        <v>1302</v>
-      </c>
-      <c r="F208" s="10">
-        <v>0</v>
-      </c>
-      <c r="G208" s="10">
-        <v>0</v>
-      </c>
-      <c r="H208" s="60">
-        <v>0</v>
-      </c>
-      <c r="I208" s="60">
-        <v>0</v>
-      </c>
-      <c r="J208" s="60">
-        <v>0</v>
-      </c>
-      <c r="K208" s="60">
-        <v>0</v>
-      </c>
-      <c r="L208" s="60" t="s">
-        <v>1303</v>
-      </c>
-      <c r="M208" s="60">
-        <v>0</v>
-      </c>
-      <c r="N208" s="60">
-        <v>0</v>
-      </c>
-      <c r="O208" s="60">
-        <v>0</v>
-      </c>
-      <c r="P208" s="60">
-        <v>0</v>
-      </c>
-      <c r="Q208" s="60">
-        <v>0</v>
-      </c>
-      <c r="R208" s="60">
-        <v>0</v>
-      </c>
-      <c r="S208" s="60">
-        <v>0</v>
-      </c>
-      <c r="T208" s="60">
-        <v>0</v>
+        <v>1294</v>
+      </c>
+      <c r="E208" s="79" t="s">
+        <v>1364</v>
+      </c>
+      <c r="F208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="G208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="H208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="I208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="J208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="K208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="L208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="M208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="N208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="O208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="P208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="Q208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="R208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="S208" s="79" t="s">
+        <v>495</v>
+      </c>
+      <c r="T208" s="79" t="s">
+        <v>495</v>
       </c>
       <c r="V208" s="6" t="s">
-        <v>1561</v>
+        <v>1584</v>
       </c>
       <c r="W208" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PF8', 'PF8', 'PAÑOS FIJOS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['OBS', 'OBS', 'OBSERVACIONES  ', 'observa',  ,  ,  ,  ,  ,  , ' ',  ,  ,  ,  ,  ,  ,  ,  ], </v>
+      </c>
+      <c r="AB208" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>['OBS', 'OBS', 'OBSERVACIONES  ', 0, 'observa'],</v>
       </c>
     </row>
     <row r="209" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30379,13 +30399,13 @@
         <v>203</v>
       </c>
       <c r="B209" s="78" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="C209" s="78" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="D209" s="92" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="E209" s="37" t="s">
         <v>1302</v>
@@ -30436,11 +30456,11 @@
         <v>0</v>
       </c>
       <c r="V209" s="6" t="s">
-        <v>1562</v>
+        <v>1561</v>
       </c>
       <c r="W209" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PF8C', 'PF8C', 'PAÑOS FIJOS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PF8', 'PF8', 'PAÑOS FIJOS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="210" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30448,13 +30468,13 @@
         <v>204</v>
       </c>
       <c r="B210" s="78" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="C210" s="78" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="D210" s="92" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="E210" s="37" t="s">
         <v>1302</v>
@@ -30505,11 +30525,11 @@
         <v>0</v>
       </c>
       <c r="V210" s="6" t="s">
-        <v>1563</v>
+        <v>1562</v>
       </c>
       <c r="W210" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PF10', 'PF10', 'PAÑOS FIJOS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PF8C', 'PF8C', 'PAÑOS FIJOS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="211" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30517,13 +30537,13 @@
         <v>205</v>
       </c>
       <c r="B211" s="78" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="C211" s="78" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="D211" s="92" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="E211" s="37" t="s">
         <v>1302</v>
@@ -30574,11 +30594,11 @@
         <v>0</v>
       </c>
       <c r="V211" s="6" t="s">
-        <v>1564</v>
+        <v>1563</v>
       </c>
       <c r="W211" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PF10C', 'PF10C', ' PAÑOS FIJOS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PF10', 'PF10', 'PAÑOS FIJOS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="212" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30586,13 +30606,13 @@
         <v>206</v>
       </c>
       <c r="B212" s="78" t="s">
-        <v>1575</v>
+        <v>1341</v>
       </c>
       <c r="C212" s="78" t="s">
-        <v>1575</v>
+        <v>1341</v>
       </c>
       <c r="D212" s="92" t="s">
-        <v>1577</v>
+        <v>1298</v>
       </c>
       <c r="E212" s="37" t="s">
         <v>1302</v>
@@ -30643,11 +30663,11 @@
         <v>0</v>
       </c>
       <c r="V212" s="6" t="s">
-        <v>1585</v>
+        <v>1564</v>
       </c>
       <c r="W212" s="18" t="str">
-        <f>CONCATENATE("['",B212,"', '",C212,"', '",D212,"', '",E212,"', ",F212,", ",G212,", ",H212,", ",I212,", ",J212,", ",K212,", '",L212,"', ",M212,", ",N212,", ",O212,", ",P212,", ",Q212,", ",R212,", ",S212,", ",T212,"], ")</f>
-        <v xml:space="preserve">['FTCV8', 'FTCV8', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">['PF10C', 'PF10C', ' PAÑOS FIJOS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="213" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30655,13 +30675,13 @@
         <v>207</v>
       </c>
       <c r="B213" s="78" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
       <c r="C213" s="78" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
       <c r="D213" s="92" t="s">
-        <v>1578</v>
+        <v>1577</v>
       </c>
       <c r="E213" s="37" t="s">
         <v>1302</v>
@@ -30712,11 +30732,11 @@
         <v>0</v>
       </c>
       <c r="V213" s="6" t="s">
-        <v>1586</v>
+        <v>1585</v>
       </c>
       <c r="W213" s="18" t="str">
         <f>CONCATENATE("['",B213,"', '",C213,"', '",D213,"', '",E213,"', ",F213,", ",G213,", ",H213,", ",I213,", ",J213,", ",K213,", '",L213,"', ",M213,", ",N213,", ",O213,", ",P213,", ",Q213,", ",R213,", ",S213,", ",T213,"], ")</f>
-        <v xml:space="preserve">['FTCV8C', 'FTCV8C', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['FTCV8', 'FTCV8', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="214" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30724,13 +30744,13 @@
         <v>208</v>
       </c>
       <c r="B214" s="78" t="s">
-        <v>1342</v>
+        <v>1576</v>
       </c>
       <c r="C214" s="78" t="s">
-        <v>1342</v>
+        <v>1576</v>
       </c>
       <c r="D214" s="92" t="s">
-        <v>1309</v>
+        <v>1578</v>
       </c>
       <c r="E214" s="37" t="s">
         <v>1302</v>
@@ -30781,11 +30801,11 @@
         <v>0</v>
       </c>
       <c r="V214" s="6" t="s">
-        <v>1587</v>
+        <v>1586</v>
       </c>
       <c r="W214" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">['FTTS10', 'FTTS10', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f>CONCATENATE("['",B214,"', '",C214,"', '",D214,"', '",E214,"', ",F214,", ",G214,", ",H214,", ",I214,", ",J214,", ",K214,", '",L214,"', ",M214,", ",N214,", ",O214,", ",P214,", ",Q214,", ",R214,", ",S214,", ",T214,"], ")</f>
+        <v xml:space="preserve">['FTCV8C', 'FTCV8C', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="215" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30793,13 +30813,13 @@
         <v>209</v>
       </c>
       <c r="B215" s="78" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="C215" s="78" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="D215" s="92" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="E215" s="37" t="s">
         <v>1302</v>
@@ -30850,11 +30870,11 @@
         <v>0</v>
       </c>
       <c r="V215" s="6" t="s">
-        <v>1588</v>
+        <v>1587</v>
       </c>
       <c r="W215" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['FTTS10C', 'FTTS10C', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['FTTS10', 'FTTS10', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="216" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30862,13 +30882,13 @@
         <v>210</v>
       </c>
       <c r="B216" s="78" t="s">
-        <v>1575</v>
+        <v>1343</v>
       </c>
       <c r="C216" s="78" t="s">
-        <v>1575</v>
+        <v>1343</v>
       </c>
       <c r="D216" s="92" t="s">
-        <v>1573</v>
+        <v>1310</v>
       </c>
       <c r="E216" s="37" t="s">
         <v>1302</v>
@@ -30919,11 +30939,11 @@
         <v>0</v>
       </c>
       <c r="V216" s="6" t="s">
-        <v>1589</v>
+        <v>1588</v>
       </c>
       <c r="W216" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['FTCV8', 'FTCV8', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['FTTS10C', 'FTTS10C', 'FRENTE TIPO SPYDER CON SOPORTE TUBULAR DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="217" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -30931,13 +30951,13 @@
         <v>211</v>
       </c>
       <c r="B217" s="78" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
       <c r="C217" s="78" t="s">
-        <v>1576</v>
+        <v>1575</v>
       </c>
       <c r="D217" s="92" t="s">
-        <v>1574</v>
+        <v>1573</v>
       </c>
       <c r="E217" s="37" t="s">
         <v>1302</v>
@@ -30988,11 +31008,11 @@
         <v>0</v>
       </c>
       <c r="V217" s="6" t="s">
-        <v>1590</v>
+        <v>1589</v>
       </c>
       <c r="W217" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['FTCV8C', 'FTCV8C', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['FTCV8', 'FTCV8', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="218" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31000,13 +31020,13 @@
         <v>212</v>
       </c>
       <c r="B218" s="78" t="s">
-        <v>1344</v>
+        <v>1576</v>
       </c>
       <c r="C218" s="78" t="s">
-        <v>1344</v>
+        <v>1576</v>
       </c>
       <c r="D218" s="92" t="s">
-        <v>1311</v>
+        <v>1574</v>
       </c>
       <c r="E218" s="37" t="s">
         <v>1302</v>
@@ -31057,11 +31077,11 @@
         <v>0</v>
       </c>
       <c r="V218" s="6" t="s">
-        <v>1591</v>
+        <v>1590</v>
       </c>
       <c r="W218" s="18" t="str">
-        <f t="shared" ref="W218:W219" si="9">CONCATENATE("['",B218,"', '",C218,"', '",D218,"', '",E218,"', ",F218,", ",G218,", ",H218,", ",I218,", ",J218,", ",K218,", '",L218,"', ",M218,", ",N218,", ",O218,", ",P218,", ",Q218,", ",R218,", ",S218,", ",T218,"], ")</f>
-        <v xml:space="preserve">['FTCV10', 'FTCV10', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">['FTCV8C', 'FTCV8C', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="219" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31069,13 +31089,13 @@
         <v>213</v>
       </c>
       <c r="B219" s="78" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="C219" s="78" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="D219" s="92" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="E219" s="37" t="s">
         <v>1302</v>
@@ -31126,11 +31146,11 @@
         <v>0</v>
       </c>
       <c r="V219" s="6" t="s">
-        <v>1592</v>
+        <v>1591</v>
       </c>
       <c r="W219" s="18" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve">['FTCV10C', 'FTCV10C', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f t="shared" ref="W219:W220" si="10">CONCATENATE("['",B219,"', '",C219,"', '",D219,"', '",E219,"', ",F219,", ",G219,", ",H219,", ",I219,", ",J219,", ",K219,", '",L219,"', ",M219,", ",N219,", ",O219,", ",P219,", ",Q219,", ",R219,", ",S219,", ",T219,"], ")</f>
+        <v xml:space="preserve">['FTCV10', 'FTCV10', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="220" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31138,13 +31158,13 @@
         <v>214</v>
       </c>
       <c r="B220" s="78" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="C220" s="78" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="D220" s="92" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="E220" s="37" t="s">
         <v>1302</v>
@@ -31195,11 +31215,11 @@
         <v>0</v>
       </c>
       <c r="V220" s="6" t="s">
-        <v>1593</v>
+        <v>1592</v>
       </c>
       <c r="W220" s="18" t="str">
-        <f t="shared" si="8"/>
-        <v xml:space="preserve">['VC2H8', 'VC2H8', 'VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f t="shared" si="10"/>
+        <v xml:space="preserve">['FTCV10C', 'FTCV10C', 'FRENTE DE VIDRIO TEMPLADO CON HERRAJES Y VIENTOS COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="221" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31207,13 +31227,13 @@
         <v>215</v>
       </c>
       <c r="B221" s="78" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="C221" s="78" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="D221" s="92" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="E221" s="37" t="s">
         <v>1302</v>
@@ -31264,11 +31284,11 @@
         <v>0</v>
       </c>
       <c r="V221" s="6" t="s">
-        <v>1594</v>
+        <v>1593</v>
       </c>
       <c r="W221" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['VC2H8C', 'VC2H8C', 'VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['VC2H8', 'VC2H8', 'VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="222" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31276,13 +31296,13 @@
         <v>216</v>
       </c>
       <c r="B222" s="78" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="C222" s="78" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="D222" s="92" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="E222" s="37" t="s">
         <v>1302</v>
@@ -31333,11 +31353,11 @@
         <v>0</v>
       </c>
       <c r="V222" s="6" t="s">
-        <v>1595</v>
+        <v>1594</v>
       </c>
       <c r="W222" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['VC4H8', 'VC4H8', 'VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['VC2H8C', 'VC2H8C', 'VENTANAS CORREDIZAS DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="223" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31345,13 +31365,13 @@
         <v>217</v>
       </c>
       <c r="B223" s="78" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="C223" s="78" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="D223" s="92" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="E223" s="37" t="s">
         <v>1302</v>
@@ -31402,11 +31422,11 @@
         <v>0</v>
       </c>
       <c r="V223" s="6" t="s">
-        <v>1596</v>
+        <v>1595</v>
       </c>
       <c r="W223" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['VC4H8C', 'VC4H8C', 'VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['VC4H8', 'VC4H8', 'VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="224" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31414,13 +31434,13 @@
         <v>218</v>
       </c>
       <c r="B224" s="78" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="C224" s="78" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="D224" s="92" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="E224" s="37" t="s">
         <v>1302</v>
@@ -31471,11 +31491,11 @@
         <v>0</v>
       </c>
       <c r="V224" s="6" t="s">
-        <v>1597</v>
+        <v>1596</v>
       </c>
       <c r="W224" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PVC2H10', 'PVC2H10', 'PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['VC4H8C', 'VC4H8C', 'VENTANAS CORREDIZAS DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 8 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="225" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31483,13 +31503,13 @@
         <v>219</v>
       </c>
       <c r="B225" s="78" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="C225" s="78" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="D225" s="92" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="E225" s="37" t="s">
         <v>1302</v>
@@ -31540,11 +31560,11 @@
         <v>0</v>
       </c>
       <c r="V225" s="6" t="s">
-        <v>1598</v>
+        <v>1597</v>
       </c>
       <c r="W225" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PVC2H10C', 'PVC2H10C', 'PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PVC2H10', 'PVC2H10', 'PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="226" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31552,13 +31572,13 @@
         <v>220</v>
       </c>
       <c r="B226" s="78" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="C226" s="78" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="D226" s="92" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="E226" s="37" t="s">
         <v>1302</v>
@@ -31609,11 +31629,11 @@
         <v>0</v>
       </c>
       <c r="V226" s="6" t="s">
-        <v>1599</v>
+        <v>1598</v>
       </c>
       <c r="W226" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PVC4H10', 'PVC4H10', 'PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PVC2H10C', 'PVC2H10C', 'PUERTA-VENTANA CORREDIZA DE 2 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="227" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31621,13 +31641,13 @@
         <v>221</v>
       </c>
       <c r="B227" s="78" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="C227" s="78" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="D227" s="92" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="E227" s="37" t="s">
         <v>1302</v>
@@ -31678,11 +31698,11 @@
         <v>0</v>
       </c>
       <c r="V227" s="6" t="s">
-        <v>1600</v>
+        <v>1599</v>
       </c>
       <c r="W227" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PVC4H10C', 'PVC4H10C', 'PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PVC4H10', 'PVC4H10', 'PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="228" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31690,13 +31710,13 @@
         <v>222</v>
       </c>
       <c r="B228" s="78" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="C228" s="78" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="D228" s="92" t="s">
-        <v>1567</v>
+        <v>1320</v>
       </c>
       <c r="E228" s="37" t="s">
         <v>1302</v>
@@ -31747,11 +31767,11 @@
         <v>0</v>
       </c>
       <c r="V228" s="6" t="s">
-        <v>1601</v>
+        <v>1600</v>
       </c>
       <c r="W228" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PB10', 'PB10', 'PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PVC4H10C', 'PVC4H10C', 'PUERTA-VENTANA CORREDIZA DE 4 HOJAS CON VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="229" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31759,13 +31779,13 @@
         <v>223</v>
       </c>
       <c r="B229" s="78" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="C229" s="78" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="D229" s="92" t="s">
-        <v>1568</v>
+        <v>1567</v>
       </c>
       <c r="E229" s="37" t="s">
         <v>1302</v>
@@ -31816,11 +31836,11 @@
         <v>0</v>
       </c>
       <c r="V229" s="6" t="s">
-        <v>1602</v>
+        <v>1601</v>
       </c>
       <c r="W229" s="18" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve">['PB10C', 'PB10C', 'PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <v xml:space="preserve">['PB10', 'PB10', 'PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="230" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31828,13 +31848,13 @@
         <v>224</v>
       </c>
       <c r="B230" s="78" t="s">
-        <v>1565</v>
+        <v>1355</v>
       </c>
       <c r="C230" s="78" t="s">
-        <v>1565</v>
+        <v>1355</v>
       </c>
       <c r="D230" s="92" t="s">
-        <v>1569</v>
+        <v>1568</v>
       </c>
       <c r="E230" s="37" t="s">
         <v>1302</v>
@@ -31885,11 +31905,11 @@
         <v>0</v>
       </c>
       <c r="V230" s="6" t="s">
-        <v>1571</v>
+        <v>1602</v>
       </c>
       <c r="W230" s="18" t="str">
-        <f t="shared" ref="W230:W231" si="10">CONCATENATE("['",B230,"', '",C230,"', '",D230,"', '",E230,"', ",F230,", ",G230,", ",H230,", ",I230,", ",J230,", ",K230,", '",L230,"', ",M230,", ",N230,", ",O230,", ",P230,", ",Q230,", ",R230,", ",S230,", ",T230,"], ")</f>
-        <v xml:space="preserve">['PB10CF', 'PB10CF', 'PUERTAS BATIENTES CON FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+        <f t="shared" si="8"/>
+        <v xml:space="preserve">['PB10C', 'PB10C', 'PUERTAS BATIENTES SIN FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>
     <row r="231" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
@@ -31897,13 +31917,13 @@
         <v>225</v>
       </c>
       <c r="B231" s="78" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="C231" s="78" t="s">
-        <v>1566</v>
+        <v>1565</v>
       </c>
       <c r="D231" s="92" t="s">
-        <v>1570</v>
+        <v>1569</v>
       </c>
       <c r="E231" s="37" t="s">
         <v>1302</v>
@@ -31954,10 +31974,79 @@
         <v>0</v>
       </c>
       <c r="V231" s="6" t="s">
+        <v>1571</v>
+      </c>
+      <c r="W231" s="18" t="str">
+        <f t="shared" ref="W231:W232" si="11">CONCATENATE("['",B231,"', '",C231,"', '",D231,"', '",E231,"', ",F231,", ",G231,", ",H231,", ",I231,", ",J231,", ",K231,", '",L231,"', ",M231,", ",N231,", ",O231,", ",P231,", ",Q231,", ",R231,", ",S231,", ",T231,"], ")</f>
+        <v xml:space="preserve">['PB10CF', 'PB10CF', 'PUERTAS BATIENTES CON FIJOS DE VIDRIO TEMPLADO INCOLORO DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
+      </c>
+    </row>
+    <row r="232" spans="1:23" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A232" s="77">
+        <v>226</v>
+      </c>
+      <c r="B232" s="78" t="s">
+        <v>1566</v>
+      </c>
+      <c r="C232" s="78" t="s">
+        <v>1566</v>
+      </c>
+      <c r="D232" s="92" t="s">
+        <v>1570</v>
+      </c>
+      <c r="E232" s="37" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F232" s="10">
+        <v>0</v>
+      </c>
+      <c r="G232" s="10">
+        <v>0</v>
+      </c>
+      <c r="H232" s="60">
+        <v>0</v>
+      </c>
+      <c r="I232" s="60">
+        <v>0</v>
+      </c>
+      <c r="J232" s="60">
+        <v>0</v>
+      </c>
+      <c r="K232" s="60">
+        <v>0</v>
+      </c>
+      <c r="L232" s="60" t="s">
+        <v>1303</v>
+      </c>
+      <c r="M232" s="60">
+        <v>0</v>
+      </c>
+      <c r="N232" s="60">
+        <v>0</v>
+      </c>
+      <c r="O232" s="60">
+        <v>0</v>
+      </c>
+      <c r="P232" s="60">
+        <v>0</v>
+      </c>
+      <c r="Q232" s="60">
+        <v>0</v>
+      </c>
+      <c r="R232" s="60">
+        <v>0</v>
+      </c>
+      <c r="S232" s="60">
+        <v>0</v>
+      </c>
+      <c r="T232" s="60">
+        <v>0</v>
+      </c>
+      <c r="V232" s="6" t="s">
         <v>1572</v>
       </c>
-      <c r="W231" s="18" t="str">
-        <f t="shared" si="10"/>
+      <c r="W232" s="18" t="str">
+        <f t="shared" si="11"/>
         <v xml:space="preserve">['PB10CFC', 'PB10CFC', 'PUERTAS BATIENTES CON FIJOS DE VIDRIO TEMPLADO COLOR DE 10 mm DE ESPESOR ', 'Pza(s).', 0, 0, 0, 0, 0, 0, 'Datos para proforma', 0, 0, 0, 0, 0, 0, 0, 0], </v>
       </c>
     </row>

</xml_diff>